<commit_message>
feat: Enhance financial engine with comprehensive debt service coverage ratios (DSCR, LLCR), equity NPV, and refined cash flow calculations.
</commit_message>
<xml_diff>
--- a/outputs/financial_output.xlsx
+++ b/outputs/financial_output.xlsx
@@ -88,8 +88,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -531,11 +531,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
@@ -550,14 +550,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hydropower Station — Hydropower (Run-of-River)</t>
+          <t>Solar PV Plant — 50 MW — Solar PV (Utility-Scale)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:24:14</t>
+          <t>Generated: 2026-03-08 22:45:02</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Hydropower Station</t>
+          <t>Solar PV Plant — 50 MW</t>
         </is>
       </c>
     </row>
@@ -590,7 +590,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Hydropower (Run-of-River)</t>
+          <t>Solar PV (Utility-Scale)</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>22.0%</t>
         </is>
       </c>
     </row>
@@ -624,7 +624,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>$125,000,000</t>
+          <t>$45,000,000</t>
         </is>
       </c>
     </row>
@@ -636,7 +636,7 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>$1,200,000</t>
+          <t>$650,000</t>
         </is>
       </c>
     </row>
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13">
@@ -670,95 +670,143 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>$55.33</t>
+          <t>$53.91</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>NPV (USD)</t>
+          <t>Project NPV (USD)</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>$-45,548,625</t>
+          <t>$10,967,700</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>FIRR (Financial)</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>5.50%</t>
+          <t>Equity NPV (USD)</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>$16,949,798</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>EIRR (Economic)</t>
+          <t>FIRR (Project)</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>11.54%</t>
+          <t>10.66%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Simple Payback (years)</t>
+          <t>EIRR (Economic)</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>19.8</t>
+          <t>12.53%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>Discounted Payback (years)</t>
+          <t>Simple Payback (years)</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>8.8</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Benefit-Cost Ratio</t>
+          <t>Discounted Payback (years)</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>0.813</t>
+          <t>15.5</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
+          <t>Benefit-Cost Ratio</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>1.178</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
           <t>Equity IRR</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>13.30%</t>
-        </is>
-      </c>
-    </row>
-    <row r="22"/>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>17.52%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Minimum DSCR</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>1.52</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Average DSCR</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>1.61</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>LLCR</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>1.60</t>
+        </is>
+      </c>
+    </row>
+    <row r="26"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
@@ -778,7 +826,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
@@ -800,7 +848,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:24:14</t>
+          <t>Generated: 2026-03-08 22:45:02</t>
         </is>
       </c>
     </row>
@@ -821,7 +869,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Hydropower Station</t>
+          <t>Solar PV Plant — 50 MW</t>
         </is>
       </c>
     </row>
@@ -833,7 +881,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Hydropower (Run-of-River)</t>
+          <t>Solar PV (Utility-Scale)</t>
         </is>
       </c>
     </row>
@@ -855,7 +903,7 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>22.0%</t>
         </is>
       </c>
     </row>
@@ -867,7 +915,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>219,000</t>
+          <t>96,360</t>
         </is>
       </c>
     </row>
@@ -878,7 +926,7 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12"/>
@@ -898,7 +946,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>$125,000,000</t>
+          <t>$45,000,000</t>
         </is>
       </c>
     </row>
@@ -910,55 +958,55 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>$1,200,000</t>
+          <t>$650,000</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Civil Works &amp; Dam</t>
+          <t xml:space="preserve">  Modules &amp; Inverters</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>$60,000,000</t>
+          <t>$25,000,000</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Turbines &amp; Generators</t>
+          <t xml:space="preserve">  Balance of System</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>$30,000,000</t>
+          <t>$10,000,000</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Electromechanical</t>
+          <t xml:space="preserve">  Engineering &amp; Development</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>$20,000,000</t>
+          <t>$5,000,000</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Engineering &amp; Contingency</t>
+          <t xml:space="preserve">  Contingency</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>$15,000,000</t>
+          <t>$5,000,000</t>
         </is>
       </c>
     </row>
@@ -1003,7 +1051,7 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>0.10%</t>
+          <t>0.50%</t>
         </is>
       </c>
     </row>
@@ -1092,24 +1140,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O46"/>
+  <dimension ref="A1:V31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="21" customWidth="1" min="11" max="11"/>
-    <col width="21" customWidth="1" min="12" max="12"/>
-    <col width="23" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="27" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="21" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="23" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="27" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1122,14 +1177,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hydropower Station — 40 year projection</t>
+          <t>Solar PV Plant — 50 MW — 25 year projection</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:24:14</t>
+          <t>Generated: 2026-03-08 22:45:02</t>
         </is>
       </c>
     </row>
@@ -1167,45 +1222,80 @@
       </c>
       <c r="G5" s="11" t="inlineStr">
         <is>
+          <t>Project Cost Basis</t>
+        </is>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
           <t>Debt Service</t>
         </is>
       </c>
-      <c r="H5" s="11" t="inlineStr">
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>Interest</t>
+        </is>
+      </c>
+      <c r="J5" s="11" t="inlineStr">
+        <is>
+          <t>Principal Repayment</t>
+        </is>
+      </c>
+      <c r="K5" s="11" t="inlineStr">
+        <is>
+          <t>CFADS</t>
+        </is>
+      </c>
+      <c r="L5" s="11" t="inlineStr">
         <is>
           <t>Depreciation</t>
         </is>
       </c>
-      <c r="I5" s="11" t="inlineStr">
-        <is>
-          <t>Tax</t>
-        </is>
-      </c>
-      <c r="J5" s="11" t="inlineStr">
+      <c r="M5" s="11" t="inlineStr">
+        <is>
+          <t>Project Tax</t>
+        </is>
+      </c>
+      <c r="N5" s="11" t="inlineStr">
+        <is>
+          <t>Equity Tax</t>
+        </is>
+      </c>
+      <c r="O5" s="11" t="inlineStr">
         <is>
           <t>Net Cash Flow</t>
         </is>
       </c>
-      <c r="K5" s="11" t="inlineStr">
+      <c r="P5" s="11" t="inlineStr">
         <is>
           <t>Economic Cash Flow</t>
         </is>
       </c>
-      <c r="L5" s="11" t="inlineStr">
+      <c r="Q5" s="11" t="inlineStr">
         <is>
           <t>Equity Cash Flow</t>
         </is>
       </c>
-      <c r="M5" s="11" t="inlineStr">
+      <c r="R5" s="11" t="inlineStr">
+        <is>
+          <t>Outstanding Debt</t>
+        </is>
+      </c>
+      <c r="S5" s="11" t="inlineStr">
+        <is>
+          <t>DSCR</t>
+        </is>
+      </c>
+      <c r="T5" s="11" t="inlineStr">
         <is>
           <t>Cumulative Cash Flow</t>
         </is>
       </c>
-      <c r="N5" s="11" t="inlineStr">
+      <c r="U5" s="11" t="inlineStr">
         <is>
           <t>Discounted CF</t>
         </is>
       </c>
-      <c r="O5" s="11" t="inlineStr">
+      <c r="V5" s="11" t="inlineStr">
         <is>
           <t>Cumulative Discounted CF</t>
         </is>
@@ -1240,22 +1330,43 @@
         <v>0</v>
       </c>
       <c r="J6" s="12" t="n">
-        <v>-125000000</v>
+        <v>0</v>
       </c>
       <c r="K6" s="12" t="n">
-        <v>-125000000</v>
+        <v>0</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>-37500000.00000001</v>
+        <v>0</v>
       </c>
       <c r="M6" s="12" t="n">
-        <v>-125000000</v>
+        <v>0</v>
       </c>
       <c r="N6" s="12" t="n">
-        <v>-125000000</v>
+        <v>0</v>
       </c>
       <c r="O6" s="12" t="n">
-        <v>-125000000</v>
+        <v>-45000000</v>
+      </c>
+      <c r="P6" s="12" t="n">
+        <v>-45000000</v>
+      </c>
+      <c r="Q6" s="12" t="n">
+        <v>-13500000</v>
+      </c>
+      <c r="R6" s="12" t="n">
+        <v>31500000</v>
+      </c>
+      <c r="S6" s="12" t="n">
+        <v/>
+      </c>
+      <c r="T6" s="12" t="n">
+        <v>-45000000</v>
+      </c>
+      <c r="U6" s="12" t="n">
+        <v>-45000000</v>
+      </c>
+      <c r="V6" s="12" t="n">
+        <v>-45000000</v>
       </c>
     </row>
     <row r="7">
@@ -1263,46 +1374,67 @@
         <v>1</v>
       </c>
       <c r="B7" s="13" t="n">
-        <v>219000</v>
+        <v>96360</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>65</v>
       </c>
       <c r="D7" s="13" t="n">
-        <v>14235000</v>
+        <v>6263400</v>
       </c>
       <c r="E7" s="13" t="n">
-        <v>1200000</v>
+        <v>650000</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>11566241.85</v>
+        <v>4566007.06</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>9009241.85</v>
+        <v>1322680</v>
       </c>
       <c r="H7" s="13" t="n">
-        <v>6250000</v>
+        <v>3243327.06</v>
       </c>
       <c r="I7" s="13" t="n">
-        <v>1357000</v>
+        <v>1890000</v>
       </c>
       <c r="J7" s="13" t="n">
-        <v>2668758.15</v>
+        <v>1353327.06</v>
       </c>
       <c r="K7" s="13" t="n">
-        <v>13035000</v>
+        <v>4940720</v>
       </c>
       <c r="L7" s="13" t="n">
-        <v>2668758.15</v>
+        <v>2250000</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>-122331241.85</v>
+        <v>672680</v>
       </c>
       <c r="N7" s="13" t="n">
-        <v>2471072.36</v>
+        <v>294680</v>
       </c>
       <c r="O7" s="13" t="n">
-        <v>-122528927.64</v>
+        <v>4940720</v>
+      </c>
+      <c r="P7" s="13" t="n">
+        <v>5613400</v>
+      </c>
+      <c r="Q7" s="13" t="n">
+        <v>2075392.94</v>
+      </c>
+      <c r="R7" s="13" t="n">
+        <v>30146672.94</v>
+      </c>
+      <c r="S7" s="13" t="n">
+        <v>1.523</v>
+      </c>
+      <c r="T7" s="13" t="n">
+        <v>-40059280</v>
+      </c>
+      <c r="U7" s="13" t="n">
+        <v>4574740.74</v>
+      </c>
+      <c r="V7" s="13" t="n">
+        <v>-40425259.26</v>
       </c>
     </row>
     <row r="8">
@@ -1310,46 +1442,67 @@
         <v>2</v>
       </c>
       <c r="B8" s="12" t="n">
-        <v>218781</v>
+        <v>95878</v>
       </c>
       <c r="C8" s="12" t="n">
         <v>65.97</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>14434076.47</v>
+        <v>6325564.24</v>
       </c>
       <c r="E8" s="12" t="n">
-        <v>1224000</v>
+        <v>663000</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>11625257.14</v>
+        <v>4588839.91</v>
       </c>
       <c r="G8" s="12" t="n">
-        <v>9009241.85</v>
+        <v>1345512.85</v>
       </c>
       <c r="H8" s="12" t="n">
-        <v>6250000</v>
+        <v>3243327.06</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>1392015.29</v>
+        <v>1808800.38</v>
       </c>
       <c r="J8" s="12" t="n">
-        <v>2808819.33</v>
+        <v>1434526.69</v>
       </c>
       <c r="K8" s="12" t="n">
-        <v>13210076.47</v>
+        <v>4980051.4</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>2808819.33</v>
+        <v>2250000</v>
       </c>
       <c r="M8" s="12" t="n">
-        <v>-119522422.51</v>
+        <v>682512.85</v>
       </c>
       <c r="N8" s="12" t="n">
-        <v>2408109.85</v>
+        <v>320752.77</v>
       </c>
       <c r="O8" s="12" t="n">
-        <v>-120120817.78</v>
+        <v>4980051.4</v>
+      </c>
+      <c r="P8" s="12" t="n">
+        <v>5662564.24</v>
+      </c>
+      <c r="Q8" s="12" t="n">
+        <v>2098484.41</v>
+      </c>
+      <c r="R8" s="12" t="n">
+        <v>28712146.25</v>
+      </c>
+      <c r="S8" s="12" t="n">
+        <v>1.535</v>
+      </c>
+      <c r="T8" s="12" t="n">
+        <v>-35079228.6</v>
+      </c>
+      <c r="U8" s="12" t="n">
+        <v>4269591.39</v>
+      </c>
+      <c r="V8" s="12" t="n">
+        <v>-36155667.87</v>
       </c>
     </row>
     <row r="9">
@@ -1357,46 +1510,67 @@
         <v>3</v>
       </c>
       <c r="B9" s="13" t="n">
-        <v>218562</v>
+        <v>95399</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>66.95999999999999</v>
       </c>
       <c r="D9" s="13" t="n">
-        <v>14635937.03</v>
+        <v>6388345.47</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>1248480</v>
+        <v>676260</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>11685213.25</v>
+        <v>4612004.16</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>9009241.85</v>
+        <v>1368677.09</v>
       </c>
       <c r="H9" s="13" t="n">
-        <v>6250000</v>
+        <v>3243327.06</v>
       </c>
       <c r="I9" s="13" t="n">
-        <v>1427491.41</v>
+        <v>1722728.77</v>
       </c>
       <c r="J9" s="13" t="n">
-        <v>2950723.78</v>
+        <v>1520598.29</v>
       </c>
       <c r="K9" s="13" t="n">
-        <v>13387457.03</v>
+        <v>5019668.38</v>
       </c>
       <c r="L9" s="13" t="n">
-        <v>2950723.78</v>
+        <v>2250000</v>
       </c>
       <c r="M9" s="13" t="n">
-        <v>-116571698.73</v>
+        <v>692417.09</v>
       </c>
       <c r="N9" s="13" t="n">
-        <v>2342379.67</v>
+        <v>347871.34</v>
       </c>
       <c r="O9" s="13" t="n">
-        <v>-117778438.11</v>
+        <v>5019668.38</v>
+      </c>
+      <c r="P9" s="13" t="n">
+        <v>5712085.47</v>
+      </c>
+      <c r="Q9" s="13" t="n">
+        <v>2120887.07</v>
+      </c>
+      <c r="R9" s="13" t="n">
+        <v>27191547.96</v>
+      </c>
+      <c r="S9" s="13" t="n">
+        <v>1.548</v>
+      </c>
+      <c r="T9" s="13" t="n">
+        <v>-30059560.23</v>
+      </c>
+      <c r="U9" s="13" t="n">
+        <v>3984774.6</v>
+      </c>
+      <c r="V9" s="13" t="n">
+        <v>-32170893.27</v>
       </c>
     </row>
     <row r="10">
@@ -1404,46 +1578,67 @@
         <v>4</v>
       </c>
       <c r="B10" s="12" t="n">
-        <v>218344</v>
+        <v>94922</v>
       </c>
       <c r="C10" s="12" t="n">
         <v>67.97</v>
       </c>
       <c r="D10" s="12" t="n">
-        <v>14840620.61</v>
+        <v>6451749.8</v>
       </c>
       <c r="E10" s="12" t="n">
-        <v>1273449.6</v>
+        <v>689785.2</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>11746125.65</v>
+        <v>4635505.18</v>
       </c>
       <c r="G10" s="12" t="n">
-        <v>9009241.85</v>
+        <v>1392178.12</v>
       </c>
       <c r="H10" s="12" t="n">
-        <v>6250000</v>
+        <v>3243327.06</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>1463434.2</v>
+        <v>1631492.88</v>
       </c>
       <c r="J10" s="12" t="n">
-        <v>3094494.97</v>
+        <v>1611834.19</v>
       </c>
       <c r="K10" s="12" t="n">
-        <v>13567171.01</v>
+        <v>5059571.68</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>3094494.97</v>
+        <v>2250000</v>
       </c>
       <c r="M10" s="12" t="n">
-        <v>-113477203.77</v>
+        <v>702392.92</v>
       </c>
       <c r="N10" s="12" t="n">
-        <v>2274546.18</v>
+        <v>376094.34</v>
       </c>
       <c r="O10" s="12" t="n">
-        <v>-115503891.93</v>
+        <v>5059571.68</v>
+      </c>
+      <c r="P10" s="12" t="n">
+        <v>5761964.6</v>
+      </c>
+      <c r="Q10" s="12" t="n">
+        <v>2142543.19</v>
+      </c>
+      <c r="R10" s="12" t="n">
+        <v>25579713.77</v>
+      </c>
+      <c r="S10" s="12" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="T10" s="12" t="n">
+        <v>-24999988.55</v>
+      </c>
+      <c r="U10" s="12" t="n">
+        <v>3718936.23</v>
+      </c>
+      <c r="V10" s="12" t="n">
+        <v>-28451957.05</v>
       </c>
     </row>
     <row r="11">
@@ -1451,46 +1646,67 @@
         <v>5</v>
       </c>
       <c r="B11" s="13" t="n">
-        <v>218125</v>
+        <v>94447</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>68.98999999999999</v>
       </c>
       <c r="D11" s="13" t="n">
-        <v>15048166.69</v>
+        <v>6515783.42</v>
       </c>
       <c r="E11" s="13" t="n">
-        <v>1298918.59</v>
+        <v>703580.9</v>
       </c>
       <c r="F11" s="13" t="n">
-        <v>11808010.06</v>
+        <v>4659348.47</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>9009241.85</v>
+        <v>1416021.41</v>
       </c>
       <c r="H11" s="13" t="n">
-        <v>6250000</v>
+        <v>3243327.06</v>
       </c>
       <c r="I11" s="13" t="n">
-        <v>1499849.62</v>
+        <v>1534782.83</v>
       </c>
       <c r="J11" s="13" t="n">
-        <v>3240156.63</v>
+        <v>1708544.24</v>
       </c>
       <c r="K11" s="13" t="n">
-        <v>13749248.1</v>
+        <v>5099762.01</v>
       </c>
       <c r="L11" s="13" t="n">
-        <v>3240156.63</v>
+        <v>2250000</v>
       </c>
       <c r="M11" s="13" t="n">
-        <v>-110237047.13</v>
+        <v>712440.5</v>
       </c>
       <c r="N11" s="13" t="n">
-        <v>2205196.16</v>
+        <v>405483.94</v>
       </c>
       <c r="O11" s="13" t="n">
-        <v>-113298695.77</v>
+        <v>5099762.01</v>
+      </c>
+      <c r="P11" s="13" t="n">
+        <v>5812202.51</v>
+      </c>
+      <c r="Q11" s="13" t="n">
+        <v>2163391.51</v>
+      </c>
+      <c r="R11" s="13" t="n">
+        <v>23871169.53</v>
+      </c>
+      <c r="S11" s="13" t="n">
+        <v>1.572</v>
+      </c>
+      <c r="T11" s="13" t="n">
+        <v>-19900226.54</v>
+      </c>
+      <c r="U11" s="13" t="n">
+        <v>3470812.33</v>
+      </c>
+      <c r="V11" s="13" t="n">
+        <v>-24981144.72</v>
       </c>
     </row>
     <row r="12">
@@ -1498,46 +1714,67 @@
         <v>6</v>
       </c>
       <c r="B12" s="12" t="n">
-        <v>217907</v>
+        <v>93975</v>
       </c>
       <c r="C12" s="12" t="n">
         <v>70.02</v>
       </c>
       <c r="D12" s="12" t="n">
-        <v>15258615.3</v>
+        <v>6580452.57</v>
       </c>
       <c r="E12" s="12" t="n">
-        <v>1324896.96</v>
+        <v>717652.52</v>
       </c>
       <c r="F12" s="12" t="n">
-        <v>11870882.48</v>
+        <v>4683539.6</v>
       </c>
       <c r="G12" s="12" t="n">
-        <v>9009241.85</v>
+        <v>1440212.53</v>
       </c>
       <c r="H12" s="12" t="n">
-        <v>6250000</v>
+        <v>3243327.06</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>1536743.67</v>
+        <v>1432270.17</v>
       </c>
       <c r="J12" s="12" t="n">
-        <v>3387732.83</v>
+        <v>1811056.89</v>
       </c>
       <c r="K12" s="12" t="n">
-        <v>13933718.34</v>
+        <v>5140240.04</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>3387732.83</v>
+        <v>2250000</v>
       </c>
       <c r="M12" s="12" t="n">
-        <v>-106849314.3</v>
+        <v>722560.01</v>
       </c>
       <c r="N12" s="12" t="n">
-        <v>2134846.33</v>
+        <v>436105.97</v>
       </c>
       <c r="O12" s="12" t="n">
-        <v>-111163849.44</v>
+        <v>5140240.04</v>
+      </c>
+      <c r="P12" s="12" t="n">
+        <v>5862800.04</v>
+      </c>
+      <c r="Q12" s="12" t="n">
+        <v>2183367</v>
+      </c>
+      <c r="R12" s="12" t="n">
+        <v>22060112.64</v>
+      </c>
+      <c r="S12" s="12" t="n">
+        <v>1.585</v>
+      </c>
+      <c r="T12" s="12" t="n">
+        <v>-14759986.5</v>
+      </c>
+      <c r="U12" s="12" t="n">
+        <v>3239223.15</v>
+      </c>
+      <c r="V12" s="12" t="n">
+        <v>-21741921.57</v>
       </c>
     </row>
     <row r="13">
@@ -1545,46 +1782,67 @@
         <v>7</v>
       </c>
       <c r="B13" s="13" t="n">
-        <v>217689</v>
+        <v>93505</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>71.06999999999999</v>
       </c>
       <c r="D13" s="13" t="n">
-        <v>15472007.04</v>
+        <v>6645763.56</v>
       </c>
       <c r="E13" s="13" t="n">
-        <v>1351394.9</v>
+        <v>732005.5699999999</v>
       </c>
       <c r="F13" s="13" t="n">
-        <v>11934759.18</v>
+        <v>4708084.23</v>
       </c>
       <c r="G13" s="13" t="n">
-        <v>9009241.85</v>
+        <v>1464757.17</v>
       </c>
       <c r="H13" s="13" t="n">
-        <v>6250000</v>
+        <v>3243327.06</v>
       </c>
       <c r="I13" s="13" t="n">
-        <v>1574122.43</v>
+        <v>1323606.76</v>
       </c>
       <c r="J13" s="13" t="n">
-        <v>3537247.86</v>
+        <v>1919720.31</v>
       </c>
       <c r="K13" s="13" t="n">
-        <v>14120612.14</v>
+        <v>5181006.39</v>
       </c>
       <c r="L13" s="13" t="n">
-        <v>3537247.86</v>
+        <v>2250000</v>
       </c>
       <c r="M13" s="13" t="n">
-        <v>-103312066.44</v>
+        <v>732751.6</v>
       </c>
       <c r="N13" s="13" t="n">
-        <v>2063950.15</v>
+        <v>468030.25</v>
       </c>
       <c r="O13" s="13" t="n">
-        <v>-109099899.28</v>
+        <v>5181006.39</v>
+      </c>
+      <c r="P13" s="13" t="n">
+        <v>5913757.99</v>
+      </c>
+      <c r="Q13" s="13" t="n">
+        <v>2202400.68</v>
+      </c>
+      <c r="R13" s="13" t="n">
+        <v>20140392.33</v>
+      </c>
+      <c r="S13" s="13" t="n">
+        <v>1.597</v>
+      </c>
+      <c r="T13" s="13" t="n">
+        <v>-9578980.119999999</v>
+      </c>
+      <c r="U13" s="13" t="n">
+        <v>3023067.47</v>
+      </c>
+      <c r="V13" s="13" t="n">
+        <v>-18718854.1</v>
       </c>
     </row>
     <row r="14">
@@ -1592,46 +1850,67 @@
         <v>8</v>
       </c>
       <c r="B14" s="12" t="n">
-        <v>217472</v>
+        <v>93038</v>
       </c>
       <c r="C14" s="12" t="n">
         <v>72.14</v>
       </c>
       <c r="D14" s="12" t="n">
-        <v>15688383.06</v>
+        <v>6711722.76</v>
       </c>
       <c r="E14" s="12" t="n">
-        <v>1378422.8</v>
+        <v>746645.6800000001</v>
       </c>
       <c r="F14" s="12" t="n">
-        <v>11999656.7</v>
+        <v>4732988.16</v>
       </c>
       <c r="G14" s="12" t="n">
-        <v>9009241.85</v>
+        <v>1489661.1</v>
       </c>
       <c r="H14" s="12" t="n">
-        <v>6250000</v>
+        <v>3243327.06</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>1611992.05</v>
+        <v>1208423.54</v>
       </c>
       <c r="J14" s="12" t="n">
-        <v>3688726.36</v>
+        <v>2034903.52</v>
       </c>
       <c r="K14" s="12" t="n">
-        <v>14309960.26</v>
+        <v>5222061.66</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>3688726.36</v>
+        <v>2250000</v>
       </c>
       <c r="M14" s="12" t="n">
-        <v>-99623340.08</v>
+        <v>743015.42</v>
       </c>
       <c r="N14" s="12" t="n">
-        <v>1992904.08</v>
+        <v>501330.71</v>
       </c>
       <c r="O14" s="12" t="n">
-        <v>-107106995.21</v>
+        <v>5222061.66</v>
+      </c>
+      <c r="P14" s="12" t="n">
+        <v>5965077.08</v>
+      </c>
+      <c r="Q14" s="12" t="n">
+        <v>2220419.31</v>
+      </c>
+      <c r="R14" s="12" t="n">
+        <v>18105488.81</v>
+      </c>
+      <c r="S14" s="12" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="T14" s="12" t="n">
+        <v>-4356918.45</v>
+      </c>
+      <c r="U14" s="12" t="n">
+        <v>2821317.43</v>
+      </c>
+      <c r="V14" s="12" t="n">
+        <v>-15897536.68</v>
       </c>
     </row>
     <row r="15">
@@ -1639,46 +1918,67 @@
         <v>9</v>
       </c>
       <c r="B15" s="13" t="n">
-        <v>217254</v>
+        <v>92572</v>
       </c>
       <c r="C15" s="13" t="n">
         <v>73.22</v>
       </c>
       <c r="D15" s="13" t="n">
-        <v>15907785.09</v>
+        <v>6778336.61</v>
       </c>
       <c r="E15" s="13" t="n">
-        <v>1405991.26</v>
+        <v>761578.6</v>
       </c>
       <c r="F15" s="13" t="n">
-        <v>12065591.87</v>
+        <v>4758257.26</v>
       </c>
       <c r="G15" s="13" t="n">
-        <v>9009241.85</v>
+        <v>1514930.2</v>
       </c>
       <c r="H15" s="13" t="n">
-        <v>6250000</v>
+        <v>3243327.06</v>
       </c>
       <c r="I15" s="13" t="n">
-        <v>1650358.77</v>
+        <v>1086329.33</v>
       </c>
       <c r="J15" s="13" t="n">
-        <v>3842193.22</v>
+        <v>2156997.74</v>
       </c>
       <c r="K15" s="13" t="n">
-        <v>14501793.84</v>
+        <v>5263406.41</v>
       </c>
       <c r="L15" s="13" t="n">
-        <v>3842193.22</v>
+        <v>2250000</v>
       </c>
       <c r="M15" s="13" t="n">
-        <v>-95781146.86</v>
+        <v>753351.6</v>
       </c>
       <c r="N15" s="13" t="n">
-        <v>1922053.19</v>
+        <v>536085.74</v>
       </c>
       <c r="O15" s="13" t="n">
-        <v>-105184942.02</v>
+        <v>5263406.41</v>
+      </c>
+      <c r="P15" s="13" t="n">
+        <v>6016758.01</v>
+      </c>
+      <c r="Q15" s="13" t="n">
+        <v>2237345.21</v>
+      </c>
+      <c r="R15" s="13" t="n">
+        <v>15948491.07</v>
+      </c>
+      <c r="S15" s="13" t="n">
+        <v>1.623</v>
+      </c>
+      <c r="T15" s="13" t="n">
+        <v>906487.96</v>
+      </c>
+      <c r="U15" s="13" t="n">
+        <v>2633013.62</v>
+      </c>
+      <c r="V15" s="13" t="n">
+        <v>-13264523.06</v>
       </c>
     </row>
     <row r="16">
@@ -1686,46 +1986,67 @@
         <v>10</v>
       </c>
       <c r="B16" s="12" t="n">
-        <v>217037</v>
+        <v>92110</v>
       </c>
       <c r="C16" s="12" t="n">
         <v>74.31999999999999</v>
       </c>
       <c r="D16" s="12" t="n">
-        <v>16130255.47</v>
+        <v>6845611.6</v>
       </c>
       <c r="E16" s="12" t="n">
-        <v>1434111.08</v>
+        <v>776810.17</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>12132581.81</v>
+        <v>4783897.52</v>
       </c>
       <c r="G16" s="12" t="n">
-        <v>9009241.85</v>
+        <v>1540570.46</v>
       </c>
       <c r="H16" s="12" t="n">
-        <v>6250000</v>
+        <v>3243327.06</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>1689228.88</v>
+        <v>956909.46</v>
       </c>
       <c r="J16" s="12" t="n">
-        <v>3997673.66</v>
+        <v>2286417.6</v>
       </c>
       <c r="K16" s="12" t="n">
-        <v>14696144.39</v>
+        <v>5305041.14</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>3997673.66</v>
+        <v>2250000</v>
       </c>
       <c r="M16" s="12" t="n">
-        <v>-91783473.19</v>
+        <v>763760.29</v>
       </c>
       <c r="N16" s="12" t="n">
-        <v>1851696.41</v>
+        <v>572378.39</v>
       </c>
       <c r="O16" s="12" t="n">
-        <v>-103333245.61</v>
+        <v>5305041.14</v>
+      </c>
+      <c r="P16" s="12" t="n">
+        <v>6068801.43</v>
+      </c>
+      <c r="Q16" s="12" t="n">
+        <v>2253095.97</v>
+      </c>
+      <c r="R16" s="12" t="n">
+        <v>13662073.47</v>
+      </c>
+      <c r="S16" s="12" t="n">
+        <v>1.636</v>
+      </c>
+      <c r="T16" s="12" t="n">
+        <v>6211529.1</v>
+      </c>
+      <c r="U16" s="12" t="n">
+        <v>2457260.51</v>
+      </c>
+      <c r="V16" s="12" t="n">
+        <v>-10807262.54</v>
       </c>
     </row>
     <row r="17">
@@ -1733,46 +2054,67 @@
         <v>11</v>
       </c>
       <c r="B17" s="13" t="n">
-        <v>216820</v>
+        <v>91649</v>
       </c>
       <c r="C17" s="13" t="n">
         <v>75.44</v>
       </c>
       <c r="D17" s="13" t="n">
-        <v>16355837.09</v>
+        <v>6913554.3</v>
       </c>
       <c r="E17" s="13" t="n">
-        <v>1462793.3</v>
+        <v>792346.37</v>
       </c>
       <c r="F17" s="13" t="n">
-        <v>12200643.91</v>
+        <v>4809915.02</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>9009241.85</v>
+        <v>1566587.96</v>
       </c>
       <c r="H17" s="13" t="n">
-        <v>6250000</v>
+        <v>3243327.06</v>
       </c>
       <c r="I17" s="13" t="n">
-        <v>1728608.76</v>
+        <v>819724.41</v>
       </c>
       <c r="J17" s="13" t="n">
-        <v>4155193.18</v>
+        <v>2423602.66</v>
       </c>
       <c r="K17" s="13" t="n">
-        <v>14893043.79</v>
+        <v>5346966.34</v>
       </c>
       <c r="L17" s="13" t="n">
-        <v>4155193.18</v>
+        <v>2250000</v>
       </c>
       <c r="M17" s="13" t="n">
-        <v>-87628280.01000001</v>
+        <v>774241.58</v>
       </c>
       <c r="N17" s="13" t="n">
-        <v>1782091.13</v>
+        <v>610296.7</v>
       </c>
       <c r="O17" s="13" t="n">
-        <v>-101551154.47</v>
+        <v>5346966.34</v>
+      </c>
+      <c r="P17" s="13" t="n">
+        <v>6121207.92</v>
+      </c>
+      <c r="Q17" s="13" t="n">
+        <v>2267584.16</v>
+      </c>
+      <c r="R17" s="13" t="n">
+        <v>11238470.82</v>
+      </c>
+      <c r="S17" s="13" t="n">
+        <v>1.649</v>
+      </c>
+      <c r="T17" s="13" t="n">
+        <v>11558495.44</v>
+      </c>
+      <c r="U17" s="13" t="n">
+        <v>2293222.21</v>
+      </c>
+      <c r="V17" s="13" t="n">
+        <v>-8514040.33</v>
       </c>
     </row>
     <row r="18">
@@ -1780,46 +2122,67 @@
         <v>12</v>
       </c>
       <c r="B18" s="12" t="n">
-        <v>216603</v>
+        <v>91191</v>
       </c>
       <c r="C18" s="12" t="n">
         <v>76.56999999999999</v>
       </c>
       <c r="D18" s="12" t="n">
-        <v>16584573.47</v>
+        <v>6982171.32</v>
       </c>
       <c r="E18" s="12" t="n">
-        <v>1492049.17</v>
+        <v>808193.3</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>12269795.88</v>
+        <v>4836315.97</v>
       </c>
       <c r="G18" s="12" t="n">
-        <v>9009241.85</v>
+        <v>1592988.9</v>
       </c>
       <c r="H18" s="12" t="n">
-        <v>6250000</v>
+        <v>3243327.06</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>1768504.86</v>
+        <v>674308.25</v>
       </c>
       <c r="J18" s="12" t="n">
-        <v>4314777.6</v>
+        <v>2569018.82</v>
       </c>
       <c r="K18" s="12" t="n">
-        <v>15092524.3</v>
+        <v>5389182.42</v>
       </c>
       <c r="L18" s="12" t="n">
-        <v>4314777.6</v>
+        <v>2250000</v>
       </c>
       <c r="M18" s="12" t="n">
-        <v>-83313502.41</v>
+        <v>784795.6</v>
       </c>
       <c r="N18" s="12" t="n">
-        <v>1713457.55</v>
+        <v>649933.95</v>
       </c>
       <c r="O18" s="12" t="n">
-        <v>-99837696.92</v>
+        <v>5389182.42</v>
+      </c>
+      <c r="P18" s="12" t="n">
+        <v>6173978.02</v>
+      </c>
+      <c r="Q18" s="12" t="n">
+        <v>2280717</v>
+      </c>
+      <c r="R18" s="12" t="n">
+        <v>8669452</v>
+      </c>
+      <c r="S18" s="12" t="n">
+        <v>1.662</v>
+      </c>
+      <c r="T18" s="12" t="n">
+        <v>16947677.85</v>
+      </c>
+      <c r="U18" s="12" t="n">
+        <v>2140118.49</v>
+      </c>
+      <c r="V18" s="12" t="n">
+        <v>-6373921.85</v>
       </c>
     </row>
     <row r="19">
@@ -1827,46 +2190,67 @@
         <v>13</v>
       </c>
       <c r="B19" s="13" t="n">
-        <v>216386</v>
+        <v>90735</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>77.72</v>
       </c>
       <c r="D19" s="13" t="n">
-        <v>16816508.73</v>
+        <v>7051469.37</v>
       </c>
       <c r="E19" s="13" t="n">
-        <v>1521890.15</v>
+        <v>824357.17</v>
       </c>
       <c r="F19" s="13" t="n">
-        <v>12340055.72</v>
+        <v>4863106.67</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>9009241.85</v>
+        <v>1619779.61</v>
       </c>
       <c r="H19" s="13" t="n">
-        <v>6250000</v>
+        <v>3243327.06</v>
       </c>
       <c r="I19" s="13" t="n">
-        <v>1808923.72</v>
+        <v>520167.12</v>
       </c>
       <c r="J19" s="13" t="n">
-        <v>4476453.02</v>
+        <v>2723159.94</v>
       </c>
       <c r="K19" s="13" t="n">
-        <v>15294618.58</v>
+        <v>5431689.76</v>
       </c>
       <c r="L19" s="13" t="n">
-        <v>4476453.02</v>
+        <v>2250000</v>
       </c>
       <c r="M19" s="13" t="n">
-        <v>-78837049.39</v>
+        <v>795422.4399999999</v>
       </c>
       <c r="N19" s="13" t="n">
-        <v>1645982.48</v>
+        <v>691389.02</v>
       </c>
       <c r="O19" s="13" t="n">
-        <v>-98191714.44</v>
+        <v>5431689.76</v>
+      </c>
+      <c r="P19" s="13" t="n">
+        <v>6227112.21</v>
+      </c>
+      <c r="Q19" s="13" t="n">
+        <v>2292396.12</v>
+      </c>
+      <c r="R19" s="13" t="n">
+        <v>5946292.06</v>
+      </c>
+      <c r="S19" s="13" t="n">
+        <v>1.675</v>
+      </c>
+      <c r="T19" s="13" t="n">
+        <v>22379367.62</v>
+      </c>
+      <c r="U19" s="13" t="n">
+        <v>1997221.05</v>
+      </c>
+      <c r="V19" s="13" t="n">
+        <v>-4376700.79</v>
       </c>
     </row>
     <row r="20">
@@ -1874,46 +2258,67 @@
         <v>14</v>
       </c>
       <c r="B20" s="12" t="n">
-        <v>216170</v>
+        <v>90281</v>
       </c>
       <c r="C20" s="12" t="n">
         <v>78.88</v>
       </c>
       <c r="D20" s="12" t="n">
-        <v>17051687.61</v>
+        <v>7121455.21</v>
       </c>
       <c r="E20" s="12" t="n">
-        <v>1552327.96</v>
+        <v>840844.3100000001</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>12411441.73</v>
+        <v>4890293.55</v>
       </c>
       <c r="G20" s="12" t="n">
-        <v>9009241.85</v>
+        <v>1646966.49</v>
       </c>
       <c r="H20" s="12" t="n">
-        <v>6250000</v>
+        <v>3243327.06</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>1849871.93</v>
+        <v>356777.52</v>
       </c>
       <c r="J20" s="12" t="n">
-        <v>4640245.88</v>
+        <v>2886549.54</v>
       </c>
       <c r="K20" s="12" t="n">
-        <v>15499359.65</v>
+        <v>5474488.72</v>
       </c>
       <c r="L20" s="12" t="n">
-        <v>4640245.88</v>
+        <v>2250000</v>
       </c>
       <c r="M20" s="12" t="n">
-        <v>-74196803.52</v>
+        <v>806122.1800000001</v>
       </c>
       <c r="N20" s="12" t="n">
-        <v>1579822.94</v>
+        <v>734766.67</v>
       </c>
       <c r="O20" s="12" t="n">
-        <v>-96611891.5</v>
+        <v>5474488.72</v>
+      </c>
+      <c r="P20" s="12" t="n">
+        <v>6280610.9</v>
+      </c>
+      <c r="Q20" s="12" t="n">
+        <v>2302517.16</v>
+      </c>
+      <c r="R20" s="12" t="n">
+        <v>3059742.51</v>
+      </c>
+      <c r="S20" s="12" t="n">
+        <v>1.688</v>
+      </c>
+      <c r="T20" s="12" t="n">
+        <v>27853856.34</v>
+      </c>
+      <c r="U20" s="12" t="n">
+        <v>1863850.13</v>
+      </c>
+      <c r="V20" s="12" t="n">
+        <v>-2512850.66</v>
       </c>
     </row>
     <row r="21">
@@ -1921,46 +2326,67 @@
         <v>15</v>
       </c>
       <c r="B21" s="13" t="n">
-        <v>215954</v>
+        <v>89830</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>80.06</v>
       </c>
       <c r="D21" s="13" t="n">
-        <v>17290155.46</v>
+        <v>7192135.65</v>
       </c>
       <c r="E21" s="13" t="n">
-        <v>1583374.52</v>
+        <v>857661.2</v>
       </c>
       <c r="F21" s="13" t="n">
-        <v>12483972.55</v>
+        <v>4917883.15</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>9009241.85</v>
+        <v>1674556.09</v>
       </c>
       <c r="H21" s="13" t="n">
-        <v>6250000</v>
+        <v>3243327.06</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>1891356.19</v>
+        <v>183584.55</v>
       </c>
       <c r="J21" s="13" t="n">
-        <v>4806182.91</v>
+        <v>3059742.51</v>
       </c>
       <c r="K21" s="13" t="n">
-        <v>15706780.94</v>
+        <v>5517579.56</v>
       </c>
       <c r="L21" s="13" t="n">
-        <v>4806182.91</v>
+        <v>2250000</v>
       </c>
       <c r="M21" s="13" t="n">
-        <v>-69390620.61</v>
+        <v>816894.89</v>
       </c>
       <c r="N21" s="13" t="n">
-        <v>1515109.29</v>
+        <v>780177.98</v>
       </c>
       <c r="O21" s="13" t="n">
-        <v>-95096782.2</v>
+        <v>5517579.56</v>
+      </c>
+      <c r="P21" s="13" t="n">
+        <v>6334474.45</v>
+      </c>
+      <c r="Q21" s="13" t="n">
+        <v>2310969.41</v>
+      </c>
+      <c r="R21" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="S21" s="13" t="n">
+        <v>1.701</v>
+      </c>
+      <c r="T21" s="13" t="n">
+        <v>33371435.9</v>
+      </c>
+      <c r="U21" s="13" t="n">
+        <v>1739371.19</v>
+      </c>
+      <c r="V21" s="13" t="n">
+        <v>-773479.47</v>
       </c>
     </row>
     <row r="22">
@@ -1968,46 +2394,67 @@
         <v>16</v>
       </c>
       <c r="B22" s="12" t="n">
-        <v>215738</v>
+        <v>89381</v>
       </c>
       <c r="C22" s="12" t="n">
         <v>81.27</v>
       </c>
       <c r="D22" s="12" t="n">
-        <v>17531958.28</v>
+        <v>7263517.59</v>
       </c>
       <c r="E22" s="12" t="n">
-        <v>1615042.01</v>
+        <v>874814.42</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>3548425.26</v>
+        <v>1702555.05</v>
       </c>
       <c r="G22" s="12" t="n">
-        <v>0</v>
+        <v>1702555.05</v>
       </c>
       <c r="H22" s="12" t="n">
-        <v>6250000</v>
+        <v>0</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>1933383.26</v>
+        <v>0</v>
       </c>
       <c r="J22" s="12" t="n">
-        <v>13983533.02</v>
+        <v>0</v>
       </c>
       <c r="K22" s="12" t="n">
-        <v>15916916.28</v>
+        <v>5560962.54</v>
       </c>
       <c r="L22" s="12" t="n">
-        <v>13983533.02</v>
+        <v>2250000</v>
       </c>
       <c r="M22" s="12" t="n">
-        <v>-55407087.59</v>
+        <v>827740.64</v>
       </c>
       <c r="N22" s="12" t="n">
-        <v>4081659.99</v>
+        <v>827740.64</v>
       </c>
       <c r="O22" s="12" t="n">
-        <v>-91015122.20999999</v>
+        <v>5560962.54</v>
+      </c>
+      <c r="P22" s="12" t="n">
+        <v>6388703.18</v>
+      </c>
+      <c r="Q22" s="12" t="n">
+        <v>5560962.54</v>
+      </c>
+      <c r="R22" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S22" s="12" t="n">
+        <v/>
+      </c>
+      <c r="T22" s="12" t="n">
+        <v>38932398.44</v>
+      </c>
+      <c r="U22" s="12" t="n">
+        <v>1623191.96</v>
+      </c>
+      <c r="V22" s="12" t="n">
+        <v>849712.48</v>
       </c>
     </row>
     <row r="23">
@@ -2015,46 +2462,67 @@
         <v>17</v>
       </c>
       <c r="B23" s="13" t="n">
-        <v>215522</v>
+        <v>88934</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>82.48</v>
       </c>
       <c r="D23" s="13" t="n">
-        <v>17777142.72</v>
+        <v>7335608.01</v>
       </c>
       <c r="E23" s="13" t="n">
-        <v>1647342.85</v>
+        <v>892310.71</v>
       </c>
       <c r="F23" s="13" t="n">
-        <v>3623302.82</v>
+        <v>1730970.17</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0</v>
+        <v>1730970.17</v>
       </c>
       <c r="H23" s="13" t="n">
-        <v>6250000</v>
+        <v>0</v>
       </c>
       <c r="I23" s="13" t="n">
-        <v>1975959.97</v>
+        <v>0</v>
       </c>
       <c r="J23" s="13" t="n">
-        <v>14153839.9</v>
+        <v>0</v>
       </c>
       <c r="K23" s="13" t="n">
-        <v>16129799.87</v>
+        <v>5604637.84</v>
       </c>
       <c r="L23" s="13" t="n">
-        <v>14153839.9</v>
+        <v>2250000</v>
       </c>
       <c r="M23" s="13" t="n">
-        <v>-41253247.69</v>
+        <v>838659.46</v>
       </c>
       <c r="N23" s="13" t="n">
-        <v>3825343.47</v>
+        <v>838659.46</v>
       </c>
       <c r="O23" s="13" t="n">
-        <v>-87189778.73999999</v>
+        <v>5604637.84</v>
+      </c>
+      <c r="P23" s="13" t="n">
+        <v>6443297.3</v>
+      </c>
+      <c r="Q23" s="13" t="n">
+        <v>5604637.84</v>
+      </c>
+      <c r="R23" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" s="13" t="n">
+        <v/>
+      </c>
+      <c r="T23" s="13" t="n">
+        <v>44537036.28</v>
+      </c>
+      <c r="U23" s="13" t="n">
+        <v>1514759.59</v>
+      </c>
+      <c r="V23" s="13" t="n">
+        <v>2364472.07</v>
       </c>
     </row>
     <row r="24">
@@ -2062,46 +2530,67 @@
         <v>18</v>
       </c>
       <c r="B24" s="12" t="n">
-        <v>215307</v>
+        <v>88489</v>
       </c>
       <c r="C24" s="12" t="n">
         <v>83.72</v>
       </c>
       <c r="D24" s="12" t="n">
-        <v>18025756.06</v>
+        <v>7408413.92</v>
       </c>
       <c r="E24" s="12" t="n">
-        <v>1680289.7</v>
+        <v>910156.92</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>3699382.97</v>
+        <v>1759808.32</v>
       </c>
       <c r="G24" s="12" t="n">
-        <v>0</v>
+        <v>1759808.32</v>
       </c>
       <c r="H24" s="12" t="n">
-        <v>6250000</v>
+        <v>0</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>2019093.27</v>
+        <v>0</v>
       </c>
       <c r="J24" s="12" t="n">
-        <v>14326373.09</v>
+        <v>0</v>
       </c>
       <c r="K24" s="12" t="n">
-        <v>16345466.36</v>
+        <v>5648605.6</v>
       </c>
       <c r="L24" s="12" t="n">
-        <v>14326373.09</v>
+        <v>2250000</v>
       </c>
       <c r="M24" s="12" t="n">
-        <v>-26926874.6</v>
+        <v>849651.4</v>
       </c>
       <c r="N24" s="12" t="n">
-        <v>3585160.96</v>
+        <v>849651.4</v>
       </c>
       <c r="O24" s="12" t="n">
-        <v>-83604617.79000001</v>
+        <v>5648605.6</v>
+      </c>
+      <c r="P24" s="12" t="n">
+        <v>6498256.99</v>
+      </c>
+      <c r="Q24" s="12" t="n">
+        <v>5648605.6</v>
+      </c>
+      <c r="R24" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S24" s="12" t="n">
+        <v/>
+      </c>
+      <c r="T24" s="12" t="n">
+        <v>50185641.87</v>
+      </c>
+      <c r="U24" s="12" t="n">
+        <v>1413558.07</v>
+      </c>
+      <c r="V24" s="12" t="n">
+        <v>3778030.14</v>
       </c>
     </row>
     <row r="25">
@@ -2109,46 +2598,67 @@
         <v>19</v>
       </c>
       <c r="B25" s="13" t="n">
-        <v>215091</v>
+        <v>88047</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>84.98</v>
       </c>
       <c r="D25" s="13" t="n">
-        <v>18277846.26</v>
+        <v>7481942.42</v>
       </c>
       <c r="E25" s="13" t="n">
-        <v>1713895.5</v>
+        <v>928360.0600000001</v>
       </c>
       <c r="F25" s="13" t="n">
-        <v>3776685.65</v>
+        <v>1789076.53</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0</v>
+        <v>1789076.53</v>
       </c>
       <c r="H25" s="13" t="n">
-        <v>6250000</v>
+        <v>0</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>2062790.15</v>
+        <v>0</v>
       </c>
       <c r="J25" s="13" t="n">
-        <v>14501160.61</v>
+        <v>0</v>
       </c>
       <c r="K25" s="13" t="n">
-        <v>16563950.76</v>
+        <v>5692865.89</v>
       </c>
       <c r="L25" s="13" t="n">
-        <v>14501160.61</v>
+        <v>2250000</v>
       </c>
       <c r="M25" s="13" t="n">
-        <v>-12425713.99</v>
+        <v>860716.47</v>
       </c>
       <c r="N25" s="13" t="n">
-        <v>3360093.86</v>
+        <v>860716.47</v>
       </c>
       <c r="O25" s="13" t="n">
-        <v>-80244523.93000001</v>
+        <v>5692865.89</v>
+      </c>
+      <c r="P25" s="13" t="n">
+        <v>6553582.36</v>
+      </c>
+      <c r="Q25" s="13" t="n">
+        <v>5692865.89</v>
+      </c>
+      <c r="R25" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="S25" s="13" t="n">
+        <v/>
+      </c>
+      <c r="T25" s="13" t="n">
+        <v>55878507.76</v>
+      </c>
+      <c r="U25" s="13" t="n">
+        <v>1319105.71</v>
+      </c>
+      <c r="V25" s="13" t="n">
+        <v>5097135.85</v>
       </c>
     </row>
     <row r="26">
@@ -2156,46 +2666,67 @@
         <v>20</v>
       </c>
       <c r="B26" s="12" t="n">
-        <v>214876</v>
+        <v>87606</v>
       </c>
       <c r="C26" s="12" t="n">
         <v>86.25</v>
       </c>
       <c r="D26" s="12" t="n">
-        <v>18533461.94</v>
+        <v>7556200.7</v>
       </c>
       <c r="E26" s="12" t="n">
-        <v>1748173.41</v>
+        <v>946927.26</v>
       </c>
       <c r="F26" s="12" t="n">
-        <v>3855231.11</v>
+        <v>1818781.95</v>
       </c>
       <c r="G26" s="12" t="n">
-        <v>0</v>
+        <v>1818781.95</v>
       </c>
       <c r="H26" s="12" t="n">
-        <v>6250000</v>
+        <v>0</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>2107057.71</v>
+        <v>0</v>
       </c>
       <c r="J26" s="12" t="n">
-        <v>14678230.83</v>
+        <v>0</v>
       </c>
       <c r="K26" s="12" t="n">
-        <v>16785288.53</v>
+        <v>5737418.75</v>
       </c>
       <c r="L26" s="12" t="n">
-        <v>14678230.83</v>
+        <v>2250000</v>
       </c>
       <c r="M26" s="12" t="n">
-        <v>2252516.84</v>
+        <v>871854.6899999999</v>
       </c>
       <c r="N26" s="12" t="n">
-        <v>3149188.11</v>
+        <v>871854.6899999999</v>
       </c>
       <c r="O26" s="12" t="n">
-        <v>-77095335.81999999</v>
+        <v>5737418.75</v>
+      </c>
+      <c r="P26" s="12" t="n">
+        <v>6609273.44</v>
+      </c>
+      <c r="Q26" s="12" t="n">
+        <v>5737418.75</v>
+      </c>
+      <c r="R26" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S26" s="12" t="n">
+        <v/>
+      </c>
+      <c r="T26" s="12" t="n">
+        <v>61615926.52</v>
+      </c>
+      <c r="U26" s="12" t="n">
+        <v>1230952.91</v>
+      </c>
+      <c r="V26" s="12" t="n">
+        <v>6328088.75</v>
       </c>
     </row>
     <row r="27">
@@ -2203,46 +2734,67 @@
         <v>21</v>
       </c>
       <c r="B27" s="13" t="n">
-        <v>214661</v>
+        <v>87168</v>
       </c>
       <c r="C27" s="13" t="n">
         <v>87.55</v>
       </c>
       <c r="D27" s="13" t="n">
-        <v>18792652.41</v>
+        <v>7631196</v>
       </c>
       <c r="E27" s="13" t="n">
-        <v>1783136.88</v>
+        <v>965865.8100000001</v>
       </c>
       <c r="F27" s="13" t="n">
-        <v>5185039.98</v>
+        <v>2298931.84</v>
       </c>
       <c r="G27" s="13" t="n">
-        <v>0</v>
+        <v>2298931.84</v>
       </c>
       <c r="H27" s="13" t="n">
         <v>0</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>3401903.11</v>
+        <v>0</v>
       </c>
       <c r="J27" s="13" t="n">
-        <v>13607612.42</v>
+        <v>0</v>
       </c>
       <c r="K27" s="13" t="n">
-        <v>17009515.53</v>
+        <v>5332264.15</v>
       </c>
       <c r="L27" s="13" t="n">
-        <v>13607612.42</v>
+        <v>0</v>
       </c>
       <c r="M27" s="13" t="n">
-        <v>15860129.26</v>
+        <v>1333066.04</v>
       </c>
       <c r="N27" s="13" t="n">
-        <v>2703230.42</v>
+        <v>1333066.04</v>
       </c>
       <c r="O27" s="13" t="n">
-        <v>-74392105.40000001</v>
+        <v>5332264.15</v>
+      </c>
+      <c r="P27" s="13" t="n">
+        <v>6665330.19</v>
+      </c>
+      <c r="Q27" s="13" t="n">
+        <v>5332264.15</v>
+      </c>
+      <c r="R27" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="S27" s="13" t="n">
+        <v/>
+      </c>
+      <c r="T27" s="13" t="n">
+        <v>66948190.67</v>
+      </c>
+      <c r="U27" s="13" t="n">
+        <v>1059284.92</v>
+      </c>
+      <c r="V27" s="13" t="n">
+        <v>7387373.67</v>
       </c>
     </row>
     <row r="28">
@@ -2250,46 +2802,67 @@
         <v>22</v>
       </c>
       <c r="B28" s="12" t="n">
-        <v>214447</v>
+        <v>86732</v>
       </c>
       <c r="C28" s="12" t="n">
         <v>88.86</v>
       </c>
       <c r="D28" s="12" t="n">
-        <v>19055467.65</v>
+        <v>7706935.62</v>
       </c>
       <c r="E28" s="12" t="n">
-        <v>1818799.61</v>
+        <v>985183.12</v>
       </c>
       <c r="F28" s="12" t="n">
-        <v>5266133.22</v>
+        <v>2329533.62</v>
       </c>
       <c r="G28" s="12" t="n">
-        <v>0</v>
+        <v>2329533.62</v>
       </c>
       <c r="H28" s="12" t="n">
         <v>0</v>
       </c>
       <c r="I28" s="12" t="n">
-        <v>3447333.61</v>
+        <v>0</v>
       </c>
       <c r="J28" s="12" t="n">
-        <v>13789334.43</v>
+        <v>0</v>
       </c>
       <c r="K28" s="12" t="n">
-        <v>17236668.04</v>
+        <v>5377401.99</v>
       </c>
       <c r="L28" s="12" t="n">
-        <v>13789334.43</v>
+        <v>0</v>
       </c>
       <c r="M28" s="12" t="n">
-        <v>29649463.69</v>
+        <v>1344350.5</v>
       </c>
       <c r="N28" s="12" t="n">
-        <v>2536417.17</v>
+        <v>1344350.5</v>
       </c>
       <c r="O28" s="12" t="n">
-        <v>-71855688.23</v>
+        <v>5377401.99</v>
+      </c>
+      <c r="P28" s="12" t="n">
+        <v>6721752.49</v>
+      </c>
+      <c r="Q28" s="12" t="n">
+        <v>5377401.99</v>
+      </c>
+      <c r="R28" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S28" s="12" t="n">
+        <v/>
+      </c>
+      <c r="T28" s="12" t="n">
+        <v>72325592.66</v>
+      </c>
+      <c r="U28" s="12" t="n">
+        <v>989122.05</v>
+      </c>
+      <c r="V28" s="12" t="n">
+        <v>8376495.72</v>
       </c>
     </row>
     <row r="29">
@@ -2297,46 +2870,67 @@
         <v>23</v>
       </c>
       <c r="B29" s="13" t="n">
-        <v>214232</v>
+        <v>86299</v>
       </c>
       <c r="C29" s="13" t="n">
         <v>90.19</v>
       </c>
       <c r="D29" s="13" t="n">
-        <v>19321958.36</v>
+        <v>7783426.95</v>
       </c>
       <c r="E29" s="13" t="n">
-        <v>1855175.6</v>
+        <v>1004886.79</v>
       </c>
       <c r="F29" s="13" t="n">
-        <v>5348532.16</v>
+        <v>2360594.82</v>
       </c>
       <c r="G29" s="13" t="n">
-        <v>0</v>
+        <v>2360594.82</v>
       </c>
       <c r="H29" s="13" t="n">
         <v>0</v>
       </c>
       <c r="I29" s="13" t="n">
-        <v>3493356.55</v>
+        <v>0</v>
       </c>
       <c r="J29" s="13" t="n">
-        <v>13973426.21</v>
+        <v>0</v>
       </c>
       <c r="K29" s="13" t="n">
-        <v>17466782.76</v>
+        <v>5422832.13</v>
       </c>
       <c r="L29" s="13" t="n">
-        <v>13973426.21</v>
+        <v>0</v>
       </c>
       <c r="M29" s="13" t="n">
-        <v>43622889.9</v>
+        <v>1355708.03</v>
       </c>
       <c r="N29" s="13" t="n">
-        <v>2379888.06</v>
+        <v>1355708.03</v>
       </c>
       <c r="O29" s="13" t="n">
-        <v>-69475800.18000001</v>
+        <v>5422832.13</v>
+      </c>
+      <c r="P29" s="13" t="n">
+        <v>6778540.17</v>
+      </c>
+      <c r="Q29" s="13" t="n">
+        <v>5422832.13</v>
+      </c>
+      <c r="R29" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="S29" s="13" t="n">
+        <v/>
+      </c>
+      <c r="T29" s="13" t="n">
+        <v>77748424.79000001</v>
+      </c>
+      <c r="U29" s="13" t="n">
+        <v>923591.2</v>
+      </c>
+      <c r="V29" s="13" t="n">
+        <v>9300086.92</v>
       </c>
     </row>
     <row r="30">
@@ -2344,46 +2938,67 @@
         <v>24</v>
       </c>
       <c r="B30" s="12" t="n">
-        <v>214018</v>
+        <v>85867</v>
       </c>
       <c r="C30" s="12" t="n">
         <v>91.54000000000001</v>
       </c>
       <c r="D30" s="12" t="n">
-        <v>19592175.95</v>
+        <v>7860677.46</v>
       </c>
       <c r="E30" s="12" t="n">
-        <v>1892279.12</v>
+        <v>1024984.52</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5432258.48</v>
+        <v>2392123.11</v>
       </c>
       <c r="G30" s="12" t="n">
-        <v>0</v>
+        <v>2392123.11</v>
       </c>
       <c r="H30" s="12" t="n">
         <v>0</v>
       </c>
       <c r="I30" s="12" t="n">
-        <v>3539979.37</v>
+        <v>0</v>
       </c>
       <c r="J30" s="12" t="n">
-        <v>14159917.47</v>
+        <v>0</v>
       </c>
       <c r="K30" s="12" t="n">
-        <v>17699896.83</v>
+        <v>5468554.35</v>
       </c>
       <c r="L30" s="12" t="n">
-        <v>14159917.47</v>
+        <v>0</v>
       </c>
       <c r="M30" s="12" t="n">
-        <v>57782807.36</v>
+        <v>1367138.59</v>
       </c>
       <c r="N30" s="12" t="n">
-        <v>2233009.6</v>
+        <v>1367138.59</v>
       </c>
       <c r="O30" s="12" t="n">
-        <v>-67242790.58</v>
+        <v>5468554.35</v>
+      </c>
+      <c r="P30" s="12" t="n">
+        <v>6835692.94</v>
+      </c>
+      <c r="Q30" s="12" t="n">
+        <v>5468554.35</v>
+      </c>
+      <c r="R30" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S30" s="12" t="n">
+        <v/>
+      </c>
+      <c r="T30" s="12" t="n">
+        <v>83216979.15000001</v>
+      </c>
+      <c r="U30" s="12" t="n">
+        <v>862387.4</v>
+      </c>
+      <c r="V30" s="12" t="n">
+        <v>10162474.32</v>
       </c>
     </row>
     <row r="31">
@@ -2391,757 +3006,73 @@
         <v>25</v>
       </c>
       <c r="B31" s="13" t="n">
-        <v>213804</v>
+        <v>85438</v>
       </c>
       <c r="C31" s="13" t="n">
         <v>92.92</v>
       </c>
       <c r="D31" s="13" t="n">
-        <v>19866172.53</v>
+        <v>7938694.69</v>
       </c>
       <c r="E31" s="13" t="n">
-        <v>1930124.7</v>
+        <v>1045484.21</v>
       </c>
       <c r="F31" s="13" t="n">
-        <v>5517334.27</v>
+        <v>2424126.31</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0</v>
+        <v>2424126.31</v>
       </c>
       <c r="H31" s="13" t="n">
         <v>0</v>
       </c>
       <c r="I31" s="13" t="n">
-        <v>3587209.57</v>
+        <v>0</v>
       </c>
       <c r="J31" s="13" t="n">
-        <v>14348838.27</v>
+        <v>0</v>
       </c>
       <c r="K31" s="13" t="n">
-        <v>17936047.83</v>
+        <v>5514568.38</v>
       </c>
       <c r="L31" s="13" t="n">
-        <v>14348838.27</v>
+        <v>0</v>
       </c>
       <c r="M31" s="13" t="n">
-        <v>72131645.63</v>
+        <v>1378642.1</v>
       </c>
       <c r="N31" s="13" t="n">
-        <v>2095187.3</v>
+        <v>1378642.1</v>
       </c>
       <c r="O31" s="13" t="n">
-        <v>-65147603.27</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="12" t="n">
-        <v>26</v>
-      </c>
-      <c r="B32" s="12" t="n">
-        <v>213590</v>
-      </c>
-      <c r="C32" s="12" t="n">
-        <v>94.31</v>
-      </c>
-      <c r="D32" s="12" t="n">
-        <v>20144000.96</v>
-      </c>
-      <c r="E32" s="12" t="n">
-        <v>1968727.19</v>
-      </c>
-      <c r="F32" s="12" t="n">
-        <v>5603781.95</v>
-      </c>
-      <c r="G32" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H32" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I32" s="12" t="n">
-        <v>3635054.75</v>
-      </c>
-      <c r="J32" s="12" t="n">
-        <v>14540219.01</v>
-      </c>
-      <c r="K32" s="12" t="n">
-        <v>18175273.76</v>
-      </c>
-      <c r="L32" s="12" t="n">
-        <v>14540219.01</v>
-      </c>
-      <c r="M32" s="12" t="n">
-        <v>86671864.64</v>
-      </c>
-      <c r="N32" s="12" t="n">
-        <v>1965863.26</v>
-      </c>
-      <c r="O32" s="12" t="n">
-        <v>-63181740.02</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="13" t="n">
-        <v>27</v>
-      </c>
-      <c r="B33" s="13" t="n">
-        <v>213377</v>
-      </c>
-      <c r="C33" s="13" t="n">
-        <v>95.73</v>
-      </c>
-      <c r="D33" s="13" t="n">
-        <v>20425714.81</v>
-      </c>
-      <c r="E33" s="13" t="n">
-        <v>2008101.74</v>
-      </c>
-      <c r="F33" s="13" t="n">
-        <v>5691624.35</v>
-      </c>
-      <c r="G33" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H33" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I33" s="13" t="n">
-        <v>3683522.61</v>
-      </c>
-      <c r="J33" s="13" t="n">
-        <v>14734090.46</v>
-      </c>
-      <c r="K33" s="13" t="n">
-        <v>18417613.07</v>
-      </c>
-      <c r="L33" s="13" t="n">
-        <v>14734090.46</v>
-      </c>
-      <c r="M33" s="13" t="n">
-        <v>101405955.1</v>
-      </c>
-      <c r="N33" s="13" t="n">
-        <v>1844513.91</v>
-      </c>
-      <c r="O33" s="13" t="n">
-        <v>-61337226.11</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="12" t="n">
-        <v>28</v>
-      </c>
-      <c r="B34" s="12" t="n">
-        <v>213163</v>
-      </c>
-      <c r="C34" s="12" t="n">
-        <v>97.16</v>
-      </c>
-      <c r="D34" s="12" t="n">
-        <v>20711368.43</v>
-      </c>
-      <c r="E34" s="12" t="n">
-        <v>2048263.77</v>
-      </c>
-      <c r="F34" s="12" t="n">
-        <v>5780884.7</v>
-      </c>
-      <c r="G34" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H34" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I34" s="12" t="n">
-        <v>3732620.93</v>
-      </c>
-      <c r="J34" s="12" t="n">
-        <v>14930483.73</v>
-      </c>
-      <c r="K34" s="12" t="n">
-        <v>18663104.66</v>
-      </c>
-      <c r="L34" s="12" t="n">
-        <v>14930483.73</v>
-      </c>
-      <c r="M34" s="12" t="n">
-        <v>116336438.82</v>
-      </c>
-      <c r="N34" s="12" t="n">
-        <v>1730647.92</v>
-      </c>
-      <c r="O34" s="12" t="n">
-        <v>-59606578.19</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="13" t="n">
-        <v>29</v>
-      </c>
-      <c r="B35" s="13" t="n">
-        <v>212950</v>
-      </c>
-      <c r="C35" s="13" t="n">
-        <v>98.62</v>
-      </c>
-      <c r="D35" s="13" t="n">
-        <v>21001016.92</v>
-      </c>
-      <c r="E35" s="13" t="n">
-        <v>2089229.05</v>
-      </c>
-      <c r="F35" s="13" t="n">
-        <v>5871586.62</v>
-      </c>
-      <c r="G35" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I35" s="13" t="n">
-        <v>3782357.57</v>
-      </c>
-      <c r="J35" s="13" t="n">
-        <v>15129430.3</v>
-      </c>
-      <c r="K35" s="13" t="n">
-        <v>18911787.87</v>
-      </c>
-      <c r="L35" s="13" t="n">
-        <v>15129430.3</v>
-      </c>
-      <c r="M35" s="13" t="n">
-        <v>131465869.12</v>
-      </c>
-      <c r="N35" s="13" t="n">
-        <v>1623804.22</v>
-      </c>
-      <c r="O35" s="13" t="n">
-        <v>-57982773.97</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="12" t="n">
-        <v>30</v>
-      </c>
-      <c r="B36" s="12" t="n">
-        <v>212737</v>
-      </c>
-      <c r="C36" s="12" t="n">
-        <v>100.1</v>
-      </c>
-      <c r="D36" s="12" t="n">
-        <v>21294716.14</v>
-      </c>
-      <c r="E36" s="12" t="n">
-        <v>2131013.63</v>
-      </c>
-      <c r="F36" s="12" t="n">
-        <v>5963754.13</v>
-      </c>
-      <c r="G36" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H36" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I36" s="12" t="n">
-        <v>3832740.5</v>
-      </c>
-      <c r="J36" s="12" t="n">
-        <v>15330962.01</v>
-      </c>
-      <c r="K36" s="12" t="n">
-        <v>19163702.51</v>
-      </c>
-      <c r="L36" s="12" t="n">
-        <v>15330962.01</v>
-      </c>
-      <c r="M36" s="12" t="n">
-        <v>146796831.13</v>
-      </c>
-      <c r="N36" s="12" t="n">
-        <v>1523550.11</v>
-      </c>
-      <c r="O36" s="12" t="n">
-        <v>-56459223.86</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="13" t="n">
-        <v>31</v>
-      </c>
-      <c r="B37" s="13" t="n">
-        <v>212524</v>
-      </c>
-      <c r="C37" s="13" t="n">
-        <v>101.6</v>
-      </c>
-      <c r="D37" s="13" t="n">
-        <v>21592522.74</v>
-      </c>
-      <c r="E37" s="13" t="n">
-        <v>2173633.9</v>
-      </c>
-      <c r="F37" s="13" t="n">
-        <v>6057411.67</v>
-      </c>
-      <c r="G37" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H37" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I37" s="13" t="n">
-        <v>3883777.77</v>
-      </c>
-      <c r="J37" s="13" t="n">
-        <v>15535111.08</v>
-      </c>
-      <c r="K37" s="13" t="n">
-        <v>19418888.84</v>
-      </c>
-      <c r="L37" s="13" t="n">
-        <v>15535111.08</v>
-      </c>
-      <c r="M37" s="13" t="n">
-        <v>162331942.21</v>
-      </c>
-      <c r="N37" s="13" t="n">
-        <v>1429479.54</v>
-      </c>
-      <c r="O37" s="13" t="n">
-        <v>-55029744.33</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="12" t="n">
-        <v>32</v>
-      </c>
-      <c r="B38" s="12" t="n">
-        <v>212312</v>
-      </c>
-      <c r="C38" s="12" t="n">
-        <v>103.12</v>
-      </c>
-      <c r="D38" s="12" t="n">
-        <v>21894494.18</v>
-      </c>
-      <c r="E38" s="12" t="n">
-        <v>2217106.58</v>
-      </c>
-      <c r="F38" s="12" t="n">
-        <v>6152584.1</v>
-      </c>
-      <c r="G38" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H38" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I38" s="12" t="n">
-        <v>3935477.52</v>
-      </c>
-      <c r="J38" s="12" t="n">
-        <v>15741910.08</v>
-      </c>
-      <c r="K38" s="12" t="n">
-        <v>19677387.6</v>
-      </c>
-      <c r="L38" s="12" t="n">
-        <v>15741910.08</v>
-      </c>
-      <c r="M38" s="12" t="n">
-        <v>178073852.28</v>
-      </c>
-      <c r="N38" s="12" t="n">
-        <v>1341211.45</v>
-      </c>
-      <c r="O38" s="12" t="n">
-        <v>-53688532.88</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="13" t="n">
-        <v>33</v>
-      </c>
-      <c r="B39" s="13" t="n">
-        <v>212100</v>
-      </c>
-      <c r="C39" s="13" t="n">
-        <v>104.67</v>
-      </c>
-      <c r="D39" s="13" t="n">
-        <v>22200688.68</v>
-      </c>
-      <c r="E39" s="13" t="n">
-        <v>2261448.71</v>
-      </c>
-      <c r="F39" s="13" t="n">
-        <v>6249296.7</v>
-      </c>
-      <c r="G39" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H39" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I39" s="13" t="n">
-        <v>3987847.99</v>
-      </c>
-      <c r="J39" s="13" t="n">
-        <v>15951391.97</v>
-      </c>
-      <c r="K39" s="13" t="n">
-        <v>19939239.97</v>
-      </c>
-      <c r="L39" s="13" t="n">
-        <v>15951391.97</v>
-      </c>
-      <c r="M39" s="13" t="n">
-        <v>194025244.26</v>
-      </c>
-      <c r="N39" s="13" t="n">
-        <v>1258388.25</v>
-      </c>
-      <c r="O39" s="13" t="n">
-        <v>-52430144.62</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="12" t="n">
-        <v>34</v>
-      </c>
-      <c r="B40" s="12" t="n">
-        <v>211887</v>
-      </c>
-      <c r="C40" s="12" t="n">
-        <v>106.24</v>
-      </c>
-      <c r="D40" s="12" t="n">
-        <v>22511165.31</v>
-      </c>
-      <c r="E40" s="12" t="n">
-        <v>2306677.68</v>
-      </c>
-      <c r="F40" s="12" t="n">
-        <v>6347575.21</v>
-      </c>
-      <c r="G40" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H40" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I40" s="12" t="n">
-        <v>4040897.52</v>
-      </c>
-      <c r="J40" s="12" t="n">
-        <v>16163590.1</v>
-      </c>
-      <c r="K40" s="12" t="n">
-        <v>20204487.62</v>
-      </c>
-      <c r="L40" s="12" t="n">
-        <v>16163590.1</v>
-      </c>
-      <c r="M40" s="12" t="n">
-        <v>210188834.35</v>
-      </c>
-      <c r="N40" s="12" t="n">
-        <v>1180674.39</v>
-      </c>
-      <c r="O40" s="12" t="n">
-        <v>-51249470.24</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="13" t="n">
-        <v>35</v>
-      </c>
-      <c r="B41" s="13" t="n">
-        <v>211676</v>
-      </c>
-      <c r="C41" s="13" t="n">
-        <v>107.83</v>
-      </c>
-      <c r="D41" s="13" t="n">
-        <v>22825983.95</v>
-      </c>
-      <c r="E41" s="13" t="n">
-        <v>2352811.24</v>
-      </c>
-      <c r="F41" s="13" t="n">
-        <v>6447445.78</v>
-      </c>
-      <c r="G41" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H41" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I41" s="13" t="n">
-        <v>4094634.54</v>
-      </c>
-      <c r="J41" s="13" t="n">
-        <v>16378538.17</v>
-      </c>
-      <c r="K41" s="13" t="n">
-        <v>20473172.72</v>
-      </c>
-      <c r="L41" s="13" t="n">
-        <v>16378538.17</v>
-      </c>
-      <c r="M41" s="13" t="n">
-        <v>226567372.53</v>
-      </c>
-      <c r="N41" s="13" t="n">
-        <v>1107754.94</v>
-      </c>
-      <c r="O41" s="13" t="n">
-        <v>-50141715.3</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="12" t="n">
-        <v>36</v>
-      </c>
-      <c r="B42" s="12" t="n">
-        <v>211464</v>
-      </c>
-      <c r="C42" s="12" t="n">
-        <v>109.45</v>
-      </c>
-      <c r="D42" s="12" t="n">
-        <v>23145205.34</v>
-      </c>
-      <c r="E42" s="12" t="n">
-        <v>2399867.46</v>
-      </c>
-      <c r="F42" s="12" t="n">
-        <v>6548935.04</v>
-      </c>
-      <c r="G42" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H42" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I42" s="12" t="n">
-        <v>4149067.58</v>
-      </c>
-      <c r="J42" s="12" t="n">
-        <v>16596270.3</v>
-      </c>
-      <c r="K42" s="12" t="n">
-        <v>20745337.88</v>
-      </c>
-      <c r="L42" s="12" t="n">
-        <v>16596270.3</v>
-      </c>
-      <c r="M42" s="12" t="n">
-        <v>243163642.83</v>
-      </c>
-      <c r="N42" s="12" t="n">
-        <v>1039334.4</v>
-      </c>
-      <c r="O42" s="12" t="n">
-        <v>-49102380.9</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="13" t="n">
-        <v>37</v>
-      </c>
-      <c r="B43" s="13" t="n">
-        <v>211252</v>
-      </c>
-      <c r="C43" s="13" t="n">
-        <v>111.09</v>
-      </c>
-      <c r="D43" s="13" t="n">
-        <v>23468891.04</v>
-      </c>
-      <c r="E43" s="13" t="n">
-        <v>2447864.81</v>
-      </c>
-      <c r="F43" s="13" t="n">
-        <v>6652070.06</v>
-      </c>
-      <c r="G43" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H43" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I43" s="13" t="n">
-        <v>4204205.24</v>
-      </c>
-      <c r="J43" s="13" t="n">
-        <v>16816820.98</v>
-      </c>
-      <c r="K43" s="13" t="n">
-        <v>21021026.22</v>
-      </c>
-      <c r="L43" s="13" t="n">
-        <v>16816820.98</v>
-      </c>
-      <c r="M43" s="13" t="n">
-        <v>259980463.81</v>
-      </c>
-      <c r="N43" s="13" t="n">
-        <v>975135.46</v>
-      </c>
-      <c r="O43" s="13" t="n">
-        <v>-48127245.44</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="12" t="n">
-        <v>38</v>
-      </c>
-      <c r="B44" s="12" t="n">
-        <v>211041</v>
-      </c>
-      <c r="C44" s="12" t="n">
-        <v>112.76</v>
-      </c>
-      <c r="D44" s="12" t="n">
-        <v>23797103.48</v>
-      </c>
-      <c r="E44" s="12" t="n">
-        <v>2496822.11</v>
-      </c>
-      <c r="F44" s="12" t="n">
-        <v>6756878.38</v>
-      </c>
-      <c r="G44" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H44" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I44" s="12" t="n">
-        <v>4260056.27</v>
-      </c>
-      <c r="J44" s="12" t="n">
-        <v>17040225.1</v>
-      </c>
-      <c r="K44" s="12" t="n">
-        <v>21300281.37</v>
-      </c>
-      <c r="L44" s="12" t="n">
-        <v>17040225.1</v>
-      </c>
-      <c r="M44" s="12" t="n">
-        <v>277020688.9</v>
-      </c>
-      <c r="N44" s="12" t="n">
-        <v>914897.87</v>
-      </c>
-      <c r="O44" s="12" t="n">
-        <v>-47212347.57</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="13" t="n">
-        <v>39</v>
-      </c>
-      <c r="B45" s="13" t="n">
-        <v>210830</v>
-      </c>
-      <c r="C45" s="13" t="n">
-        <v>114.45</v>
-      </c>
-      <c r="D45" s="13" t="n">
-        <v>24129905.97</v>
-      </c>
-      <c r="E45" s="13" t="n">
-        <v>2546758.55</v>
-      </c>
-      <c r="F45" s="13" t="n">
-        <v>6863388.03</v>
-      </c>
-      <c r="G45" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H45" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I45" s="13" t="n">
-        <v>4316629.48</v>
-      </c>
-      <c r="J45" s="13" t="n">
-        <v>17266517.94</v>
-      </c>
-      <c r="K45" s="13" t="n">
-        <v>21583147.42</v>
-      </c>
-      <c r="L45" s="13" t="n">
-        <v>17266517.94</v>
-      </c>
-      <c r="M45" s="13" t="n">
-        <v>294287206.84</v>
-      </c>
-      <c r="N45" s="13" t="n">
-        <v>858377.45</v>
-      </c>
-      <c r="O45" s="13" t="n">
-        <v>-46353970.11</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="12" t="n">
-        <v>40</v>
-      </c>
-      <c r="B46" s="12" t="n">
-        <v>210619</v>
-      </c>
-      <c r="C46" s="12" t="n">
-        <v>116.17</v>
-      </c>
-      <c r="D46" s="12" t="n">
-        <v>24467362.7</v>
-      </c>
-      <c r="E46" s="12" t="n">
-        <v>2597693.72</v>
-      </c>
-      <c r="F46" s="12" t="n">
-        <v>6971627.52</v>
-      </c>
-      <c r="G46" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H46" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I46" s="12" t="n">
-        <v>4373933.8</v>
-      </c>
-      <c r="J46" s="12" t="n">
-        <v>17495735.19</v>
-      </c>
-      <c r="K46" s="12" t="n">
-        <v>21869668.98</v>
-      </c>
-      <c r="L46" s="12" t="n">
-        <v>17495735.19</v>
-      </c>
-      <c r="M46" s="12" t="n">
-        <v>311782942.02</v>
-      </c>
-      <c r="N46" s="12" t="n">
-        <v>805345.02</v>
-      </c>
-      <c r="O46" s="12" t="n">
-        <v>-45548625.1</v>
+        <v>5514568.38</v>
+      </c>
+      <c r="P31" s="13" t="n">
+        <v>6893210.48</v>
+      </c>
+      <c r="Q31" s="13" t="n">
+        <v>5514568.38</v>
+      </c>
+      <c r="R31" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="S31" s="13" t="n">
+        <v/>
+      </c>
+      <c r="T31" s="13" t="n">
+        <v>88731547.53</v>
+      </c>
+      <c r="U31" s="13" t="n">
+        <v>805225.72</v>
+      </c>
+      <c r="V31" s="13" t="n">
+        <v>10967700.04</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A2:O2"/>
+    <mergeCell ref="A2:V2"/>
+    <mergeCell ref="A1:V1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3157,7 +3088,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
@@ -3179,7 +3110,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:24:14</t>
+          <t>Generated: 2026-03-08 22:45:02</t>
         </is>
       </c>
     </row>
@@ -3200,7 +3131,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>$55.33</t>
+          <t>$53.91</t>
         </is>
       </c>
     </row>
@@ -3216,7 +3147,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>$142,967,237</t>
+          <t>$53,238,123</t>
         </is>
       </c>
     </row>
@@ -3228,7 +3159,7 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>$125,000,000</t>
+          <t>$45,000,000</t>
         </is>
       </c>
     </row>
@@ -3240,7 +3171,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>$17,967,237</t>
+          <t>$8,238,123</t>
         </is>
       </c>
     </row>
@@ -3260,7 +3191,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>2,584,132</t>
+          <t>987,611</t>
         </is>
       </c>
     </row>
@@ -3280,7 +3211,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>$48.37</t>
+          <t>$45.56</t>
         </is>
       </c>
     </row>
@@ -3292,7 +3223,7 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>$6.95</t>
+          <t>$8.34</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3285,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:24:14</t>
+          <t>Generated: 2026-03-08 22:45:02</t>
         </is>
       </c>
     </row>
@@ -3469,19 +3400,19 @@
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>45.65</v>
+        <v>44.79</v>
       </c>
       <c r="C6" s="12" t="n">
-        <v>50.49</v>
+        <v>49.35</v>
       </c>
       <c r="D6" s="12" t="n">
-        <v>55.33</v>
+        <v>53.91</v>
       </c>
       <c r="E6" s="12" t="n">
-        <v>60.16</v>
+        <v>58.46</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>65</v>
+        <v>63.02</v>
       </c>
       <c r="G6" s="12" t="n">
         <v/>
@@ -3551,19 +3482,19 @@
         <v/>
       </c>
       <c r="G7" s="13" t="n">
-        <v>41.11</v>
+        <v>43.36</v>
       </c>
       <c r="H7" s="13" t="n">
-        <v>45.64</v>
+        <v>46.73</v>
       </c>
       <c r="I7" s="13" t="n">
-        <v>55.33</v>
+        <v>53.91</v>
       </c>
       <c r="J7" s="13" t="n">
-        <v>65.62</v>
+        <v>61.56</v>
       </c>
       <c r="K7" s="13" t="n">
-        <v>76.31999999999999</v>
+        <v>69.61</v>
       </c>
       <c r="L7" s="13" t="n">
         <v/>
@@ -3633,19 +3564,19 @@
         <v/>
       </c>
       <c r="L8" s="12" t="n">
-        <v>55.33</v>
+        <v>53.91</v>
       </c>
       <c r="M8" s="12" t="n">
-        <v>55.33</v>
+        <v>53.91</v>
       </c>
       <c r="N8" s="12" t="n">
-        <v>55.33</v>
+        <v>53.91</v>
       </c>
       <c r="O8" s="12" t="n">
-        <v>55.33</v>
+        <v>53.91</v>
       </c>
       <c r="P8" s="12" t="n">
-        <v>55.33</v>
+        <v>53.91</v>
       </c>
       <c r="Q8" s="12" t="n">
         <v/>
@@ -3715,19 +3646,19 @@
         <v/>
       </c>
       <c r="Q9" s="13" t="n">
-        <v>153.68</v>
+        <v>65.89</v>
       </c>
       <c r="R9" s="13" t="n">
-        <v>138.31</v>
+        <v>59.3</v>
       </c>
       <c r="S9" s="13" t="n">
-        <v>125.74</v>
+        <v>53.91</v>
       </c>
       <c r="T9" s="13" t="n">
-        <v>115.26</v>
+        <v>49.41</v>
       </c>
       <c r="U9" s="13" t="n">
-        <v>106.39</v>
+        <v>45.61</v>
       </c>
     </row>
     <row r="10">
@@ -3737,19 +3668,19 @@
         </is>
       </c>
       <c r="B10" s="12" t="n">
-        <v>53.93</v>
+        <v>52.24</v>
       </c>
       <c r="C10" s="12" t="n">
-        <v>54.63</v>
+        <v>53.07</v>
       </c>
       <c r="D10" s="12" t="n">
-        <v>55.33</v>
+        <v>53.91</v>
       </c>
       <c r="E10" s="12" t="n">
-        <v>56.02</v>
+        <v>54.74</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>56.72</v>
+        <v>55.57</v>
       </c>
       <c r="G10" s="12" t="n">
         <v/>
@@ -3816,26 +3747,26 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="13" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
-    <col width="16" customWidth="1" min="18" max="18"/>
-    <col width="15" customWidth="1" min="19" max="19"/>
-    <col width="16" customWidth="1" min="20" max="20"/>
-    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3855,7 +3786,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:24:14</t>
+          <t>Generated: 2026-03-08 22:45:02</t>
         </is>
       </c>
     </row>
@@ -3970,19 +3901,19 @@
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>-7580279.24</v>
+        <v>19084066.78</v>
       </c>
       <c r="C6" s="12" t="n">
-        <v>-26564452.16</v>
+        <v>15025883.41</v>
       </c>
       <c r="D6" s="12" t="n">
-        <v>-45548625.1</v>
+        <v>10967700.05</v>
       </c>
       <c r="E6" s="12" t="n">
-        <v>-64532798.03</v>
+        <v>6909516.68</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>-83516970.95999999</v>
+        <v>2851333.31</v>
       </c>
       <c r="G6" s="12" t="n">
         <v/>
@@ -4052,19 +3983,19 @@
         <v/>
       </c>
       <c r="G7" s="13" t="n">
-        <v>13022609.32</v>
+        <v>29442698.87</v>
       </c>
       <c r="H7" s="13" t="n">
-        <v>-11460798.07</v>
+        <v>22350887.82</v>
       </c>
       <c r="I7" s="13" t="n">
-        <v>-45548625.1</v>
+        <v>10967700.05</v>
       </c>
       <c r="J7" s="13" t="n">
-        <v>-67000424.83</v>
+        <v>2371512.26</v>
       </c>
       <c r="K7" s="13" t="n">
-        <v>-80989322.67</v>
+        <v>-4243547.51</v>
       </c>
       <c r="L7" s="13" t="n">
         <v/>
@@ -4134,19 +4065,19 @@
         <v/>
       </c>
       <c r="L8" s="12" t="n">
-        <v>-94369207.93000001</v>
+        <v>-6921540.67</v>
       </c>
       <c r="M8" s="12" t="n">
-        <v>-69958916.54000001</v>
+        <v>2023079.69</v>
       </c>
       <c r="N8" s="12" t="n">
-        <v>-45548625.1</v>
+        <v>10967700.05</v>
       </c>
       <c r="O8" s="12" t="n">
-        <v>-21138333.68</v>
+        <v>19912320.4</v>
       </c>
       <c r="P8" s="12" t="n">
-        <v>3271957.72</v>
+        <v>28856940.75</v>
       </c>
       <c r="Q8" s="12" t="n">
         <v/>
@@ -4216,19 +4147,19 @@
         <v/>
       </c>
       <c r="Q9" s="13" t="n">
-        <v>-150964799.43</v>
+        <v>396785.06</v>
       </c>
       <c r="R9" s="13" t="n">
-        <v>-143381668.89</v>
+        <v>5682242.55</v>
       </c>
       <c r="S9" s="13" t="n">
-        <v>-135808939.3</v>
+        <v>10967700.05</v>
       </c>
       <c r="T9" s="13" t="n">
-        <v>-128506164.17</v>
+        <v>16253157.53</v>
       </c>
       <c r="U9" s="13" t="n">
-        <v>-121717586.17</v>
+        <v>21538615.01</v>
       </c>
     </row>
     <row r="10">
@@ -4238,19 +4169,19 @@
         </is>
       </c>
       <c r="B10" s="12" t="n">
-        <v>-42673867.11</v>
+        <v>12285799.77</v>
       </c>
       <c r="C10" s="12" t="n">
-        <v>-44111246.11</v>
+        <v>11626749.92</v>
       </c>
       <c r="D10" s="12" t="n">
-        <v>-45548625.1</v>
+        <v>10967700.05</v>
       </c>
       <c r="E10" s="12" t="n">
-        <v>-46986004.1</v>
+        <v>10308650.18</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>-48423383.11</v>
+        <v>9649600.32</v>
       </c>
       <c r="G10" s="12" t="n">
         <v/>
@@ -4356,7 +4287,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:24:14</t>
+          <t>Generated: 2026-03-08 22:45:02</t>
         </is>
       </c>
     </row>
@@ -4471,19 +4402,19 @@
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>0.07489999999999999</v>
+        <v>0.1356</v>
       </c>
       <c r="C6" s="12" t="n">
-        <v>0.064</v>
+        <v>0.1197</v>
       </c>
       <c r="D6" s="12" t="n">
-        <v>0.055</v>
+        <v>0.1066</v>
       </c>
       <c r="E6" s="12" t="n">
-        <v>0.0474</v>
+        <v>0.0955</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>0.0409</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="G6" s="12" t="n">
         <v/>
@@ -4553,19 +4484,19 @@
         <v/>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.055</v>
+        <v>0.1066</v>
       </c>
       <c r="H7" s="13" t="n">
-        <v>0.055</v>
+        <v>0.1066</v>
       </c>
       <c r="I7" s="13" t="n">
-        <v>0.055</v>
+        <v>0.1066</v>
       </c>
       <c r="J7" s="13" t="n">
-        <v>0.055</v>
+        <v>0.1066</v>
       </c>
       <c r="K7" s="13" t="n">
-        <v>0.055</v>
+        <v>0.1066</v>
       </c>
       <c r="L7" s="13" t="n">
         <v/>
@@ -4635,19 +4566,19 @@
         <v/>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.025</v>
+        <v>0.0617</v>
       </c>
       <c r="M8" s="12" t="n">
-        <v>0.0406</v>
+        <v>0.0851</v>
       </c>
       <c r="N8" s="12" t="n">
-        <v>0.055</v>
+        <v>0.1066</v>
       </c>
       <c r="O8" s="12" t="n">
-        <v>0.06859999999999999</v>
+        <v>0.1269</v>
       </c>
       <c r="P8" s="12" t="n">
-        <v>0.08169999999999999</v>
+        <v>0.1463</v>
       </c>
       <c r="Q8" s="12" t="n">
         <v/>
@@ -4717,19 +4648,19 @@
         <v/>
       </c>
       <c r="Q9" s="13" t="n">
-        <v>-0.0211</v>
+        <v>0.081</v>
       </c>
       <c r="R9" s="13" t="n">
-        <v>-0.0137</v>
+        <v>0.0941</v>
       </c>
       <c r="S9" s="13" t="n">
-        <v>-0.0069</v>
+        <v>0.1066</v>
       </c>
       <c r="T9" s="13" t="n">
-        <v>-0.0008</v>
+        <v>0.1187</v>
       </c>
       <c r="U9" s="13" t="n">
-        <v>0.0047</v>
+        <v>0.1305</v>
       </c>
     </row>
     <row r="10">
@@ -4739,19 +4670,19 @@
         </is>
       </c>
       <c r="B10" s="12" t="n">
-        <v>0.0567</v>
+        <v>0.1096</v>
       </c>
       <c r="C10" s="12" t="n">
-        <v>0.0558</v>
+        <v>0.1081</v>
       </c>
       <c r="D10" s="12" t="n">
-        <v>0.055</v>
+        <v>0.1066</v>
       </c>
       <c r="E10" s="12" t="n">
-        <v>0.0542</v>
+        <v>0.1051</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.0533</v>
+        <v>0.1036</v>
       </c>
       <c r="G10" s="12" t="n">
         <v/>
@@ -4857,7 +4788,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:24:14</t>
+          <t>Generated: 2026-03-08 22:45:02</t>
         </is>
       </c>
     </row>
@@ -4972,19 +4903,19 @@
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>0.1427</v>
+        <v>0.1599</v>
       </c>
       <c r="C6" s="12" t="n">
-        <v>0.1277</v>
+        <v>0.1409</v>
       </c>
       <c r="D6" s="12" t="n">
-        <v>0.1154</v>
+        <v>0.1253</v>
       </c>
       <c r="E6" s="12" t="n">
-        <v>0.1053</v>
+        <v>0.1122</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>0.09660000000000001</v>
+        <v>0.101</v>
       </c>
       <c r="G6" s="12" t="n">
         <v/>
@@ -5054,19 +4985,19 @@
         <v/>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.1154</v>
+        <v>0.1253</v>
       </c>
       <c r="H7" s="13" t="n">
-        <v>0.1154</v>
+        <v>0.1253</v>
       </c>
       <c r="I7" s="13" t="n">
-        <v>0.1154</v>
+        <v>0.1253</v>
       </c>
       <c r="J7" s="13" t="n">
-        <v>0.1154</v>
+        <v>0.1253</v>
       </c>
       <c r="K7" s="13" t="n">
-        <v>0.1154</v>
+        <v>0.1253</v>
       </c>
       <c r="L7" s="13" t="n">
         <v/>
@@ -5136,19 +5067,19 @@
         <v/>
       </c>
       <c r="L8" s="12" t="n">
-        <v>0.0761</v>
+        <v>0.0726</v>
       </c>
       <c r="M8" s="12" t="n">
-        <v>0.0963</v>
+        <v>0.1</v>
       </c>
       <c r="N8" s="12" t="n">
-        <v>0.1154</v>
+        <v>0.1253</v>
       </c>
       <c r="O8" s="12" t="n">
-        <v>0.1339</v>
+        <v>0.1494</v>
       </c>
       <c r="P8" s="12" t="n">
-        <v>0.152</v>
+        <v>0.1727</v>
       </c>
       <c r="Q8" s="12" t="n">
         <v/>
@@ -5218,19 +5149,19 @@
         <v/>
       </c>
       <c r="Q9" s="13" t="n">
-        <v>0.0231</v>
+        <v>0.09520000000000001</v>
       </c>
       <c r="R9" s="13" t="n">
-        <v>0.0308</v>
+        <v>0.1105</v>
       </c>
       <c r="S9" s="13" t="n">
-        <v>0.038</v>
+        <v>0.1253</v>
       </c>
       <c r="T9" s="13" t="n">
-        <v>0.0448</v>
+        <v>0.1397</v>
       </c>
       <c r="U9" s="13" t="n">
-        <v>0.0512</v>
+        <v>0.1537</v>
       </c>
     </row>
     <row r="10">
@@ -5240,19 +5171,19 @@
         </is>
       </c>
       <c r="B10" s="12" t="n">
-        <v>0.1176</v>
+        <v>0.1289</v>
       </c>
       <c r="C10" s="12" t="n">
-        <v>0.1165</v>
+        <v>0.1271</v>
       </c>
       <c r="D10" s="12" t="n">
-        <v>0.1154</v>
+        <v>0.1253</v>
       </c>
       <c r="E10" s="12" t="n">
-        <v>0.1143</v>
+        <v>0.1235</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.1133</v>
+        <v>0.1218</v>
       </c>
       <c r="G10" s="12" t="n">
         <v/>
@@ -5319,10 +5250,10 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5335,7 +5266,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:24:14</t>
+          <t>Generated: 2026-03-08 22:45:02</t>
         </is>
       </c>
     </row>
@@ -5374,54 +5305,54 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>-48423383.11</v>
+        <v>9649600.32</v>
       </c>
       <c r="C5" s="12" t="n">
-        <v>-42673867.11</v>
+        <v>12285799.77</v>
       </c>
       <c r="D5" s="12" t="n">
-        <v>5749516</v>
+        <v>2636199.45</v>
       </c>
       <c r="E5" s="12" t="n">
-        <v>-45548625.1</v>
+        <v>10967700.05</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>Capacity Factor</t>
+          <t>CAPEX</t>
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>-150964799.43</v>
+        <v>2851333.31</v>
       </c>
       <c r="C6" s="13" t="n">
-        <v>-121717586.17</v>
+        <v>19084066.78</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>29247213.26</v>
+        <v>16232733.47</v>
       </c>
       <c r="E6" s="13" t="n">
-        <v>-135808939.3</v>
+        <v>10967700.05</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>CAPEX</t>
+          <t>Capacity Factor</t>
         </is>
       </c>
       <c r="B7" s="12" t="n">
-        <v>-83516970.95999999</v>
+        <v>396785.06</v>
       </c>
       <c r="C7" s="12" t="n">
-        <v>-7580279.24</v>
+        <v>21538615.01</v>
       </c>
       <c r="D7" s="12" t="n">
-        <v>75936691.72</v>
+        <v>21141829.95</v>
       </c>
       <c r="E7" s="12" t="n">
-        <v>-45548625.1</v>
+        <v>10967700.05</v>
       </c>
     </row>
     <row r="8">
@@ -5431,16 +5362,16 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>-80989322.67</v>
+        <v>-4243547.51</v>
       </c>
       <c r="C8" s="13" t="n">
-        <v>13022609.32</v>
+        <v>29442698.87</v>
       </c>
       <c r="D8" s="13" t="n">
-        <v>94011931.98999999</v>
+        <v>33686246.38</v>
       </c>
       <c r="E8" s="13" t="n">
-        <v>-45548625.1</v>
+        <v>10967700.05</v>
       </c>
     </row>
     <row r="9">
@@ -5450,16 +5381,16 @@
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>-94369207.93000001</v>
+        <v>-6921540.67</v>
       </c>
       <c r="C9" s="12" t="n">
-        <v>3271957.72</v>
+        <v>28856940.75</v>
       </c>
       <c r="D9" s="12" t="n">
-        <v>97641165.65000001</v>
+        <v>35778481.42</v>
       </c>
       <c r="E9" s="12" t="n">
-        <v>-45548625.1</v>
+        <v>10967700.05</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Introduce project management with save/load functionality and generate PDF board reports for analyses.
</commit_message>
<xml_diff>
--- a/outputs/financial_output.xlsx
+++ b/outputs/financial_output.xlsx
@@ -557,7 +557,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 22:45:02</t>
+          <t>Generated: 2026-03-08 23:08:10</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 22:45:02</t>
+          <t>Generated: 2026-03-08 23:08:10</t>
         </is>
       </c>
     </row>
@@ -1184,7 +1184,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 22:45:02</t>
+          <t>Generated: 2026-03-08 23:08:10</t>
         </is>
       </c>
     </row>
@@ -3110,7 +3110,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 22:45:02</t>
+          <t>Generated: 2026-03-08 23:08:10</t>
         </is>
       </c>
     </row>
@@ -3285,7 +3285,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 22:45:02</t>
+          <t>Generated: 2026-03-08 23:08:10</t>
         </is>
       </c>
     </row>
@@ -3786,7 +3786,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 22:45:02</t>
+          <t>Generated: 2026-03-08 23:08:10</t>
         </is>
       </c>
     </row>
@@ -4287,7 +4287,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 22:45:02</t>
+          <t>Generated: 2026-03-08 23:08:10</t>
         </is>
       </c>
     </row>
@@ -4788,7 +4788,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 22:45:02</t>
+          <t>Generated: 2026-03-08 23:08:10</t>
         </is>
       </c>
     </row>
@@ -5266,7 +5266,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 22:45:02</t>
+          <t>Generated: 2026-03-08 23:08:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Add advanced analytical capabilities for time series forecasting, renewable energy scenario planning, and financial Monte Carlo simulations.
</commit_message>
<xml_diff>
--- a/outputs/financial_output.xlsx
+++ b/outputs/financial_output.xlsx
@@ -557,7 +557,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:08:10</t>
+          <t>Generated: 2026-03-08 23:10:45</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:08:10</t>
+          <t>Generated: 2026-03-08 23:10:45</t>
         </is>
       </c>
     </row>
@@ -1184,7 +1184,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:08:10</t>
+          <t>Generated: 2026-03-08 23:10:45</t>
         </is>
       </c>
     </row>
@@ -3110,7 +3110,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:08:10</t>
+          <t>Generated: 2026-03-08 23:10:45</t>
         </is>
       </c>
     </row>
@@ -3285,7 +3285,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:08:10</t>
+          <t>Generated: 2026-03-08 23:10:45</t>
         </is>
       </c>
     </row>
@@ -3786,7 +3786,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:08:10</t>
+          <t>Generated: 2026-03-08 23:10:45</t>
         </is>
       </c>
     </row>
@@ -4287,7 +4287,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:08:10</t>
+          <t>Generated: 2026-03-08 23:10:45</t>
         </is>
       </c>
     </row>
@@ -4788,7 +4788,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:08:10</t>
+          <t>Generated: 2026-03-08 23:10:45</t>
         </is>
       </c>
     </row>
@@ -5266,7 +5266,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:08:10</t>
+          <t>Generated: 2026-03-08 23:10:45</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Add new project data, analysis history, and PDF report, and update existing scenario, financial, and regression output spreadsheets.
</commit_message>
<xml_diff>
--- a/outputs/financial_output.xlsx
+++ b/outputs/financial_output.xlsx
@@ -557,7 +557,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:10:45</t>
+          <t>Generated: 2026-03-08 23:24:35</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:10:45</t>
+          <t>Generated: 2026-03-08 23:24:35</t>
         </is>
       </c>
     </row>
@@ -1184,7 +1184,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:10:45</t>
+          <t>Generated: 2026-03-08 23:24:35</t>
         </is>
       </c>
     </row>
@@ -3110,7 +3110,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:10:45</t>
+          <t>Generated: 2026-03-08 23:24:35</t>
         </is>
       </c>
     </row>
@@ -3285,7 +3285,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:10:45</t>
+          <t>Generated: 2026-03-08 23:24:35</t>
         </is>
       </c>
     </row>
@@ -3786,7 +3786,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:10:45</t>
+          <t>Generated: 2026-03-08 23:24:35</t>
         </is>
       </c>
     </row>
@@ -4287,7 +4287,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:10:45</t>
+          <t>Generated: 2026-03-08 23:24:35</t>
         </is>
       </c>
     </row>
@@ -4788,7 +4788,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:10:45</t>
+          <t>Generated: 2026-03-08 23:24:35</t>
         </is>
       </c>
     </row>
@@ -5266,7 +5266,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:10:45</t>
+          <t>Generated: 2026-03-08 23:24:35</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Add new regression project data and report, updating scenario, financial, and regression outputs.
</commit_message>
<xml_diff>
--- a/outputs/financial_output.xlsx
+++ b/outputs/financial_output.xlsx
@@ -557,7 +557,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:24:35</t>
+          <t>Generated: 2026-03-08 23:36:12</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:24:35</t>
+          <t>Generated: 2026-03-08 23:36:12</t>
         </is>
       </c>
     </row>
@@ -1184,7 +1184,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:24:35</t>
+          <t>Generated: 2026-03-08 23:36:12</t>
         </is>
       </c>
     </row>
@@ -3110,7 +3110,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:24:35</t>
+          <t>Generated: 2026-03-08 23:36:12</t>
         </is>
       </c>
     </row>
@@ -3285,7 +3285,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:24:35</t>
+          <t>Generated: 2026-03-08 23:36:12</t>
         </is>
       </c>
     </row>
@@ -3786,7 +3786,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:24:35</t>
+          <t>Generated: 2026-03-08 23:36:12</t>
         </is>
       </c>
     </row>
@@ -4287,7 +4287,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:24:35</t>
+          <t>Generated: 2026-03-08 23:36:12</t>
         </is>
       </c>
     </row>
@@ -4788,7 +4788,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:24:35</t>
+          <t>Generated: 2026-03-08 23:36:12</t>
         </is>
       </c>
     </row>
@@ -5266,7 +5266,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-03-08 23:24:35</t>
+          <t>Generated: 2026-03-08 23:36:12</t>
         </is>
       </c>
     </row>

</xml_diff>